<commit_message>
Expand Molson Coors and Anheuser-Busch facility networks
</commit_message>
<xml_diff>
--- a/source-data/Strategic_End_User_Facilities_Bottler_Expansion_V3.xlsx
+++ b/source-data/Strategic_End_User_Facilities_Bottler_Expansion_V3.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Facilities v2" sheetId="1" r:id="R5f5029321fce4dee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Coverage" sheetId="2" r:id="R13fe13a66f644daf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope &amp; Notes" sheetId="3" r:id="R2e55d16559a04560"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coordinate Audit" sheetId="4" r:id="Re6416f6a991e461a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Facilities v2" sheetId="1" r:id="Rd6dcfc7046dd4bb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Coverage" sheetId="2" r:id="R37f1391f71bf4cda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope &amp; Notes" sheetId="3" r:id="R0e1beeef49f746e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coordinate Audit" sheetId="4" r:id="Rd4228c53efa04fb9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -53,9 +53,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">New column</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Operating / Bottler Entity separates the strategic parent from the actual company operating each production facility.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Coca-Cola approach</x:t>
@@ -325,8 +322,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="StrategicFacilitiesV2" displayName="StrategicFacilitiesV2" ref="A1:P388" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:P388"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="StrategicFacilitiesV2" displayName="StrategicFacilitiesV2" ref="A1:P405" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:P405"/>
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="Vertical"/>
     <x:tableColumn id="2" name="Ultimate Parent"/>
@@ -350,8 +347,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="BottlerCoverage" displayName="BottlerCoverage" ref="A1:F14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F14"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="BottlerCoverage" displayName="BottlerCoverage" ref="A1:F15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F15"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Vertical"/>
     <x:tableColumn id="2" name="Ultimate Parent"/>
@@ -365,8 +362,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="CoordinateAuditTable" displayName="CoordinateAuditTable" ref="A1:F388" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F388"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="CoordinateAuditTable" displayName="CoordinateAuditTable" ref="A1:F405" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F405"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Excel Row"/>
     <x:tableColumn id="2" name="Facility Name"/>
@@ -1329,42 +1326,46 @@
         <x:v>AB InBev Belgium N.V. (HQ)</x:v>
       </x:c>
       <x:c r="C17" s="2" t="str">
-        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+        <x:v>Goose Island Beer Co</x:v>
       </x:c>
       <x:c r="D17" s="2" t="str">
-        <x:v>Anheuser-Busch Brewery - Fairfield</x:v>
+        <x:v>Goose Island - Fulton Street Brewery</x:v>
       </x:c>
       <x:c r="E17" s="2" t="str">
-        <x:v>Brewery</x:v>
-      </x:c>
-      <x:c r="F17" s="2"/>
+        <x:v>Craft brewery</x:v>
+      </x:c>
+      <x:c r="F17" s="2" t="str">
+        <x:v>1800 W. Fulton St</x:v>
+      </x:c>
       <x:c r="G17" s="2" t="str">
-        <x:v>Fairfield</x:v>
+        <x:v>Chicago</x:v>
       </x:c>
       <x:c r="H17" s="2" t="str">
-        <x:v>CA</x:v>
-      </x:c>
-      <x:c r="I17" s="2"/>
+        <x:v>IL</x:v>
+      </x:c>
+      <x:c r="I17" s="2" t="str">
+        <x:v>60612</x:v>
+      </x:c>
       <x:c r="J17" s="2" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="K17" s="15" t="n">
-        <x:v>38.24936</x:v>
+        <x:v>41.85003</x:v>
       </x:c>
       <x:c r="L17" s="15" t="n">
-        <x:v>-122.03997</x:v>
+        <x:v>-87.65005</x:v>
       </x:c>
       <x:c r="M17" s="2" t="str">
-        <x:v>West</x:v>
+        <x:v>Midwest</x:v>
       </x:c>
       <x:c r="N17" s="2" t="str">
-        <x:v>Closure / sale announced - verify active status</x:v>
+        <x:v>Verified - source-supported</x:v>
       </x:c>
       <x:c r="O17" s="2" t="str">
-        <x:v>https://www.anheuser-busch.com/facilities</x:v>
+        <x:v>https://www.gooseisland.com/taproom</x:v>
       </x:c>
       <x:c r="P17" s="2" t="str">
-        <x:v>Restructuring affects this site; do not treat as active without current validation.</x:v>
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="30" hidden="1">
@@ -1375,42 +1376,46 @@
         <x:v>AB InBev Belgium N.V. (HQ)</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
-        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+        <x:v>Golden Road Brewing</x:v>
       </x:c>
       <x:c r="D18" s="2" t="str">
-        <x:v>Anheuser-Busch Brewery - Merrimack</x:v>
+        <x:v>Golden Road - Atwater Village Brewery</x:v>
       </x:c>
       <x:c r="E18" s="2" t="str">
-        <x:v>Brewery</x:v>
-      </x:c>
-      <x:c r="F18" s="2"/>
+        <x:v>Craft brewery</x:v>
+      </x:c>
+      <x:c r="F18" s="2" t="str">
+        <x:v>5410 W San Fernando Rd</x:v>
+      </x:c>
       <x:c r="G18" s="2" t="str">
-        <x:v>Merrimack</x:v>
+        <x:v>Los Angeles</x:v>
       </x:c>
       <x:c r="H18" s="2" t="str">
-        <x:v>NH</x:v>
-      </x:c>
-      <x:c r="I18" s="2"/>
+        <x:v>CA</x:v>
+      </x:c>
+      <x:c r="I18" s="2" t="str">
+        <x:v>90039</x:v>
+      </x:c>
       <x:c r="J18" s="2" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="K18" s="15" t="n">
-        <x:v>42.86509</x:v>
+        <x:v>34.05223</x:v>
       </x:c>
       <x:c r="L18" s="15" t="n">
-        <x:v>-71.4934</x:v>
+        <x:v>-118.24368</x:v>
       </x:c>
       <x:c r="M18" s="2" t="str">
-        <x:v>Northeast</x:v>
+        <x:v>West</x:v>
       </x:c>
       <x:c r="N18" s="2" t="str">
-        <x:v>Closure / sale announced - verify active status</x:v>
+        <x:v>Verified - source-supported</x:v>
       </x:c>
       <x:c r="O18" s="2" t="str">
-        <x:v>https://www.anheuser-busch.com/facilities</x:v>
+        <x:v>https://www.goldenroad.la/brewpubs</x:v>
       </x:c>
       <x:c r="P18" s="2" t="str">
-        <x:v>Restructuring affects this site; do not treat as active without current validation.</x:v>
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="30" hidden="1">
@@ -1421,42 +1426,46 @@
         <x:v>AB InBev Belgium N.V. (HQ)</x:v>
       </x:c>
       <x:c r="C19" s="2" t="str">
-        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+        <x:v>Golden Road Brewing</x:v>
       </x:c>
       <x:c r="D19" s="2" t="str">
-        <x:v>Anheuser-Busch Brewery - Newark</x:v>
+        <x:v>Golden Road - Anaheim Brewery</x:v>
       </x:c>
       <x:c r="E19" s="2" t="str">
-        <x:v>Brewery</x:v>
-      </x:c>
-      <x:c r="F19" s="2"/>
+        <x:v>Craft brewery</x:v>
+      </x:c>
+      <x:c r="F19" s="2" t="str">
+        <x:v>2210 E Orangewood Ave</x:v>
+      </x:c>
       <x:c r="G19" s="2" t="str">
-        <x:v>Newark</x:v>
+        <x:v>Anaheim</x:v>
       </x:c>
       <x:c r="H19" s="2" t="str">
-        <x:v>NJ</x:v>
-      </x:c>
-      <x:c r="I19" s="2"/>
+        <x:v>CA</x:v>
+      </x:c>
+      <x:c r="I19" s="2" t="str">
+        <x:v>92806</x:v>
+      </x:c>
       <x:c r="J19" s="2" t="str">
         <x:v>United States</x:v>
       </x:c>
       <x:c r="K19" s="15" t="n">
-        <x:v>40.73566</x:v>
+        <x:v>33.83529</x:v>
       </x:c>
       <x:c r="L19" s="15" t="n">
-        <x:v>-74.17237</x:v>
+        <x:v>-117.9145</x:v>
       </x:c>
       <x:c r="M19" s="2" t="str">
-        <x:v>Northeast</x:v>
+        <x:v>West</x:v>
       </x:c>
       <x:c r="N19" s="2" t="str">
-        <x:v>Closure / sale announced - verify active status</x:v>
+        <x:v>Verified - source-supported</x:v>
       </x:c>
       <x:c r="O19" s="2" t="str">
-        <x:v>https://www.anheuser-busch.com/facilities</x:v>
+        <x:v>https://www.goldenroad.la/brewpubs</x:v>
       </x:c>
       <x:c r="P19" s="2" t="str">
-        <x:v>Restructuring affects this site; do not treat as active without current validation.</x:v>
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="30">
@@ -1628,13 +1637,13 @@
         <x:v>Midwest</x:v>
       </x:c>
       <x:c r="N23" s="2" t="str">
-        <x:v>Current status check required</x:v>
+        <x:v>Verified current - official 2026 source</x:v>
       </x:c>
       <x:c r="O23" s="2" t="str">
-        <x:v>https://www.anheuser-busch.com/newsroom/arnold-mcc</x:v>
+        <x:v>https://www.anheuser-busch.com/newsroom/Anheuser-Busch-Invests-20-Million-in-St-Louis-Brewery</x:v>
       </x:c>
       <x:c r="P23" s="2" t="str">
-        <x:v>Network location identified; exact address/current operating status still to validate.</x:v>
+        <x:v>MCC remains a separate strategic account. Current A-B investment announcement confirms the Arnold can plant.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="30" hidden="1">
@@ -1674,13 +1683,13 @@
         <x:v>Southeast</x:v>
       </x:c>
       <x:c r="N24" s="2" t="str">
-        <x:v>Current status check required</x:v>
+        <x:v>Verified current - official 2026 source</x:v>
       </x:c>
       <x:c r="O24" s="2" t="str">
-        <x:v>https://www.anheuser-busch.com/newsroom/arnold-mcc</x:v>
+        <x:v>https://www.anheuser-busch.com/newsroom/anheuser-busch-investing-in-jacksonville-facilities-to-drive-local-economic-growth</x:v>
       </x:c>
       <x:c r="P24" s="2" t="str">
-        <x:v>Network location identified; exact address/current operating status still to validate.</x:v>
+        <x:v>MCC remains a separate strategic account. Current A-B investment announcement confirms the Jacksonville can plant.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="30" hidden="1">
@@ -1720,13 +1729,13 @@
         <x:v>West</x:v>
       </x:c>
       <x:c r="N25" s="2" t="str">
-        <x:v>Current status check required</x:v>
+        <x:v>Official network listing; current site check pending</x:v>
       </x:c>
       <x:c r="O25" s="2" t="str">
-        <x:v>https://www.anheuser-busch.com/newsroom/arnold-mcc</x:v>
+        <x:v>https://www.anheuser-busch.com/newsroom/anheuser-busch-to-invest-70-million-to-80-million-in-arnold-mo-metal-container-corp-facility</x:v>
       </x:c>
       <x:c r="P25" s="2" t="str">
-        <x:v>Network location identified; exact address/current operating status still to validate.</x:v>
+        <x:v>MCC remains a separate strategic account. Facility appears in A-B's official seven-plant MCC network listing; fresh plant-specific confirmation remains pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="30" hidden="1">
@@ -1766,13 +1775,13 @@
         <x:v>Northeast</x:v>
       </x:c>
       <x:c r="N26" s="2" t="str">
-        <x:v>Current status check required</x:v>
+        <x:v>Official network listing; current site check pending</x:v>
       </x:c>
       <x:c r="O26" s="2" t="str">
-        <x:v>https://www.anheuser-busch.com/newsroom/arnold-mcc</x:v>
+        <x:v>https://www.anheuser-busch.com/newsroom/anheuser-busch-to-invest-70-million-to-80-million-in-arnold-mo-metal-container-corp-facility</x:v>
       </x:c>
       <x:c r="P26" s="2" t="str">
-        <x:v>Network location identified; exact address/current operating status still to validate.</x:v>
+        <x:v>MCC remains a separate strategic account. Facility appears in A-B's official seven-plant MCC network listing; fresh plant-specific confirmation remains pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="30" hidden="1">
@@ -1812,13 +1821,13 @@
         <x:v>West</x:v>
       </x:c>
       <x:c r="N27" s="2" t="str">
-        <x:v>Current status check required</x:v>
+        <x:v>Official network listing; current site check pending</x:v>
       </x:c>
       <x:c r="O27" s="2" t="str">
-        <x:v>https://www.anheuser-busch.com/newsroom/arnold-mcc</x:v>
+        <x:v>https://www.anheuser-busch.com/newsroom/anheuser-busch-to-invest-70-million-to-80-million-in-arnold-mo-metal-container-corp-facility</x:v>
       </x:c>
       <x:c r="P27" s="2" t="str">
-        <x:v>Network location identified; exact address/current operating status still to validate.</x:v>
+        <x:v>MCC remains a separate strategic account. Facility appears in A-B's official seven-plant MCC network listing; fresh plant-specific confirmation remains pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="30" hidden="1">
@@ -1858,13 +1867,13 @@
         <x:v>Midwest</x:v>
       </x:c>
       <x:c r="N28" s="2" t="str">
-        <x:v>Current status check required</x:v>
+        <x:v>Official network listing; current site check pending</x:v>
       </x:c>
       <x:c r="O28" s="2" t="str">
-        <x:v>https://www.anheuser-busch.com/newsroom/arnold-mcc</x:v>
+        <x:v>https://www.anheuser-busch.com/newsroom/anheuser-busch-to-invest-70-million-to-80-million-in-arnold-mo-metal-container-corp-facility</x:v>
       </x:c>
       <x:c r="P28" s="2" t="str">
-        <x:v>Network location identified; exact address/current operating status still to validate.</x:v>
+        <x:v>MCC remains a separate strategic account. Facility appears in A-B's official seven-plant MCC network listing; fresh plant-specific confirmation remains pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="30" hidden="1">
@@ -1904,13 +1913,13 @@
         <x:v>West</x:v>
       </x:c>
       <x:c r="N29" s="2" t="str">
-        <x:v>Current status check required</x:v>
+        <x:v>Official network listing; current site check pending</x:v>
       </x:c>
       <x:c r="O29" s="2" t="str">
-        <x:v>https://www.anheuser-busch.com/newsroom/arnold-mcc</x:v>
+        <x:v>https://www.anheuser-busch.com/newsroom/anheuser-busch-to-invest-70-million-to-80-million-in-arnold-mo-metal-container-corp-facility</x:v>
       </x:c>
       <x:c r="P29" s="2" t="str">
-        <x:v>Network location identified; exact address/current operating status still to validate.</x:v>
+        <x:v>MCC remains a separate strategic account. Facility appears in A-B's official seven-plant MCC network listing; fresh plant-specific confirmation remains pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="1">
@@ -1924,19 +1933,23 @@
         <x:v>Molson Coors Beverage Company</x:v>
       </x:c>
       <x:c r="D30" s="2" t="str">
-        <x:v>Molson Coors - Golden</x:v>
+        <x:v>Molson Coors - Golden Brewery</x:v>
       </x:c>
       <x:c r="E30" s="2" t="str">
         <x:v>Brewery</x:v>
       </x:c>
-      <x:c r="F30" s="2"/>
+      <x:c r="F30" s="2" t="str">
+        <x:v>12th &amp; Ford Street</x:v>
+      </x:c>
       <x:c r="G30" s="2" t="str">
         <x:v>Golden</x:v>
       </x:c>
       <x:c r="H30" s="2" t="str">
         <x:v>CO</x:v>
       </x:c>
-      <x:c r="I30" s="2"/>
+      <x:c r="I30" s="2" t="str">
+        <x:v>80401</x:v>
+      </x:c>
       <x:c r="J30" s="2" t="str">
         <x:v>United States</x:v>
       </x:c>
@@ -1950,12 +1963,14 @@
         <x:v>West</x:v>
       </x:c>
       <x:c r="N30" s="2" t="str">
-        <x:v>Verified city - street address pending</x:v>
+        <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O30" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/</x:v>
-      </x:c>
-      <x:c r="P30" s="2"/>
+        <x:v>https://www.molsoncoors.com/our-locations/us/brewery/golden</x:v>
+      </x:c>
+      <x:c r="P30" s="2" t="str">
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="1">
       <x:c r="A31" s="2" t="str">
@@ -1968,19 +1983,23 @@
         <x:v>Molson Coors Beverage Company</x:v>
       </x:c>
       <x:c r="D31" s="2" t="str">
-        <x:v>Molson Coors - Milwaukee</x:v>
+        <x:v>Molson Coors - Milwaukee Brewery</x:v>
       </x:c>
       <x:c r="E31" s="2" t="str">
         <x:v>Brewery</x:v>
       </x:c>
-      <x:c r="F31" s="2"/>
+      <x:c r="F31" s="2" t="str">
+        <x:v>4000 W. State Street</x:v>
+      </x:c>
       <x:c r="G31" s="2" t="str">
         <x:v>Milwaukee</x:v>
       </x:c>
       <x:c r="H31" s="2" t="str">
         <x:v>WI</x:v>
       </x:c>
-      <x:c r="I31" s="2"/>
+      <x:c r="I31" s="2" t="str">
+        <x:v>53208</x:v>
+      </x:c>
       <x:c r="J31" s="2" t="str">
         <x:v>United States</x:v>
       </x:c>
@@ -1994,12 +2013,14 @@
         <x:v>Midwest</x:v>
       </x:c>
       <x:c r="N31" s="2" t="str">
-        <x:v>Verified city - street address pending</x:v>
+        <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O31" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/</x:v>
-      </x:c>
-      <x:c r="P31" s="2"/>
+        <x:v>https://www.molsoncoors.com/our-locations/us/brewery/milwaukee</x:v>
+      </x:c>
+      <x:c r="P31" s="2" t="str">
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="1">
       <x:c r="A32" s="2" t="str">
@@ -2012,19 +2033,23 @@
         <x:v>Molson Coors Beverage Company</x:v>
       </x:c>
       <x:c r="D32" s="2" t="str">
-        <x:v>Molson Coors - Albany</x:v>
+        <x:v>Molson Coors - Albany Brewery</x:v>
       </x:c>
       <x:c r="E32" s="2" t="str">
         <x:v>Brewery</x:v>
       </x:c>
-      <x:c r="F32" s="2"/>
+      <x:c r="F32" s="2" t="str">
+        <x:v>405 Cordele Road</x:v>
+      </x:c>
       <x:c r="G32" s="2" t="str">
         <x:v>Albany</x:v>
       </x:c>
       <x:c r="H32" s="2" t="str">
         <x:v>GA</x:v>
       </x:c>
-      <x:c r="I32" s="2"/>
+      <x:c r="I32" s="2" t="str">
+        <x:v>31705</x:v>
+      </x:c>
       <x:c r="J32" s="2" t="str">
         <x:v>United States</x:v>
       </x:c>
@@ -2038,12 +2063,14 @@
         <x:v>Southeast</x:v>
       </x:c>
       <x:c r="N32" s="2" t="str">
-        <x:v>Verified city - street address pending</x:v>
+        <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O32" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/</x:v>
-      </x:c>
-      <x:c r="P32" s="2"/>
+        <x:v>https://www.molsoncoors.com/our-locations/us/brewery/albany</x:v>
+      </x:c>
+      <x:c r="P32" s="2" t="str">
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="1">
       <x:c r="A33" s="2" t="str">
@@ -2056,19 +2083,23 @@
         <x:v>Molson Coors Beverage Company</x:v>
       </x:c>
       <x:c r="D33" s="2" t="str">
-        <x:v>Molson Coors - Fort Worth</x:v>
+        <x:v>Molson Coors - Fort Worth Brewery</x:v>
       </x:c>
       <x:c r="E33" s="2" t="str">
         <x:v>Brewery</x:v>
       </x:c>
-      <x:c r="F33" s="2"/>
+      <x:c r="F33" s="2" t="str">
+        <x:v>7001 South Freeway</x:v>
+      </x:c>
       <x:c r="G33" s="2" t="str">
         <x:v>Fort Worth</x:v>
       </x:c>
       <x:c r="H33" s="2" t="str">
         <x:v>TX</x:v>
       </x:c>
-      <x:c r="I33" s="2"/>
+      <x:c r="I33" s="2" t="str">
+        <x:v>76134</x:v>
+      </x:c>
       <x:c r="J33" s="2" t="str">
         <x:v>United States</x:v>
       </x:c>
@@ -2082,12 +2113,14 @@
         <x:v>South</x:v>
       </x:c>
       <x:c r="N33" s="2" t="str">
-        <x:v>Verified city - street address pending</x:v>
+        <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O33" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/</x:v>
-      </x:c>
-      <x:c r="P33" s="2"/>
+        <x:v>https://www.molsoncoors.com/our-locations/us/brewery/fort-worth</x:v>
+      </x:c>
+      <x:c r="P33" s="2" t="str">
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="1">
       <x:c r="A34" s="2" t="str">
@@ -2100,19 +2133,23 @@
         <x:v>Molson Coors Beverage Company</x:v>
       </x:c>
       <x:c r="D34" s="2" t="str">
-        <x:v>Molson Coors - Trenton</x:v>
+        <x:v>Molson Coors - Trenton Brewery</x:v>
       </x:c>
       <x:c r="E34" s="2" t="str">
         <x:v>Brewery</x:v>
       </x:c>
-      <x:c r="F34" s="2"/>
+      <x:c r="F34" s="2" t="str">
+        <x:v>2525 Wayne Madison Rd.</x:v>
+      </x:c>
       <x:c r="G34" s="2" t="str">
         <x:v>Trenton</x:v>
       </x:c>
       <x:c r="H34" s="2" t="str">
         <x:v>OH</x:v>
       </x:c>
-      <x:c r="I34" s="2"/>
+      <x:c r="I34" s="2" t="str">
+        <x:v>45067</x:v>
+      </x:c>
       <x:c r="J34" s="2" t="str">
         <x:v>United States</x:v>
       </x:c>
@@ -2126,12 +2163,14 @@
         <x:v>Ohio Valley</x:v>
       </x:c>
       <x:c r="N34" s="2" t="str">
-        <x:v>Verified city - street address pending</x:v>
+        <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O34" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/</x:v>
-      </x:c>
-      <x:c r="P34" s="2"/>
+        <x:v>https://www.molsoncoors.com/our-locations/us/brewery/trenton</x:v>
+      </x:c>
+      <x:c r="P34" s="2" t="str">
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="1">
       <x:c r="A35" s="2" t="str">
@@ -2144,19 +2183,23 @@
         <x:v>Molson Coors Beverage Company</x:v>
       </x:c>
       <x:c r="D35" s="2" t="str">
-        <x:v>Molson Coors - Elkton</x:v>
+        <x:v>Molson Coors - Shenandoah Brewery</x:v>
       </x:c>
       <x:c r="E35" s="2" t="str">
         <x:v>Brewery</x:v>
       </x:c>
-      <x:c r="F35" s="2"/>
+      <x:c r="F35" s="2" t="str">
+        <x:v>5135 S. East Side Highway</x:v>
+      </x:c>
       <x:c r="G35" s="2" t="str">
         <x:v>Elkton</x:v>
       </x:c>
       <x:c r="H35" s="2" t="str">
         <x:v>VA</x:v>
       </x:c>
-      <x:c r="I35" s="2"/>
+      <x:c r="I35" s="2" t="str">
+        <x:v>22827</x:v>
+      </x:c>
       <x:c r="J35" s="2" t="str">
         <x:v>United States</x:v>
       </x:c>
@@ -2170,12 +2213,14 @@
         <x:v>Northeast</x:v>
       </x:c>
       <x:c r="N35" s="2" t="str">
-        <x:v>Verified city - street address pending</x:v>
+        <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O35" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/</x:v>
-      </x:c>
-      <x:c r="P35" s="2"/>
+        <x:v>https://www.molsoncoors.com/our-locations/us/brewery/shenandoah</x:v>
+      </x:c>
+      <x:c r="P35" s="2" t="str">
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="1">
       <x:c r="A36" s="2" t="str">
@@ -2188,19 +2233,23 @@
         <x:v>Molson Coors Beverage Company</x:v>
       </x:c>
       <x:c r="D36" s="2" t="str">
-        <x:v>Molson Coors - Chilliwack</x:v>
+        <x:v>Molson Coors - Fraser Valley Brewery</x:v>
       </x:c>
       <x:c r="E36" s="2" t="str">
         <x:v>Brewery</x:v>
       </x:c>
-      <x:c r="F36" s="2"/>
+      <x:c r="F36" s="2" t="str">
+        <x:v>45620 Kerr Avenue</x:v>
+      </x:c>
       <x:c r="G36" s="2" t="str">
         <x:v>Chilliwack</x:v>
       </x:c>
       <x:c r="H36" s="2" t="str">
         <x:v>BC</x:v>
       </x:c>
-      <x:c r="I36" s="2"/>
+      <x:c r="I36" s="2" t="str">
+        <x:v>V2R 0Z7</x:v>
+      </x:c>
       <x:c r="J36" s="2" t="str">
         <x:v>Canada</x:v>
       </x:c>
@@ -2214,12 +2263,14 @@
         <x:v>Canada</x:v>
       </x:c>
       <x:c r="N36" s="2" t="str">
-        <x:v>Verified city - street address pending</x:v>
+        <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O36" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/</x:v>
-      </x:c>
-      <x:c r="P36" s="2"/>
+        <x:v>https://www.molsoncoors.com/our-locations/ca/brewery/fraservalley</x:v>
+      </x:c>
+      <x:c r="P36" s="2" t="str">
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="1">
       <x:c r="A37" s="2" t="str">
@@ -2232,19 +2283,23 @@
         <x:v>Molson Coors Beverage Company</x:v>
       </x:c>
       <x:c r="D37" s="2" t="str">
-        <x:v>Molson Coors - Longueuil</x:v>
+        <x:v>Molson Coors - Longueuil Brewery</x:v>
       </x:c>
       <x:c r="E37" s="2" t="str">
         <x:v>Brewery</x:v>
       </x:c>
-      <x:c r="F37" s="2"/>
+      <x:c r="F37" s="2" t="str">
+        <x:v>6125 Route De L'aeroport</x:v>
+      </x:c>
       <x:c r="G37" s="2" t="str">
-        <x:v>Longueuil</x:v>
+        <x:v>Saint-Hubert</x:v>
       </x:c>
       <x:c r="H37" s="2" t="str">
         <x:v>QC</x:v>
       </x:c>
-      <x:c r="I37" s="2"/>
+      <x:c r="I37" s="2" t="str">
+        <x:v>J3Y 8Y9</x:v>
+      </x:c>
       <x:c r="J37" s="2" t="str">
         <x:v>Canada</x:v>
       </x:c>
@@ -2258,12 +2313,14 @@
         <x:v>Canada</x:v>
       </x:c>
       <x:c r="N37" s="2" t="str">
-        <x:v>Verified city - street address pending</x:v>
+        <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O37" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/</x:v>
-      </x:c>
-      <x:c r="P37" s="2"/>
+        <x:v>https://www.molsoncoors.com/our-locations/ca/brewery/longueuil</x:v>
+      </x:c>
+      <x:c r="P37" s="2" t="str">
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="1">
       <x:c r="A38" s="2" t="str">
@@ -2276,19 +2333,23 @@
         <x:v>Molson Coors Beverage Company</x:v>
       </x:c>
       <x:c r="D38" s="2" t="str">
-        <x:v>Molson Coors - St. John's</x:v>
+        <x:v>Molson Coors - St. John's Brewery</x:v>
       </x:c>
       <x:c r="E38" s="2" t="str">
         <x:v>Brewery</x:v>
       </x:c>
-      <x:c r="F38" s="2"/>
+      <x:c r="F38" s="2" t="str">
+        <x:v>131 Circular Road</x:v>
+      </x:c>
       <x:c r="G38" s="2" t="str">
         <x:v>St. John's</x:v>
       </x:c>
       <x:c r="H38" s="2" t="str">
         <x:v>NL</x:v>
       </x:c>
-      <x:c r="I38" s="2"/>
+      <x:c r="I38" s="2" t="str">
+        <x:v>A1C 5W1</x:v>
+      </x:c>
       <x:c r="J38" s="2" t="str">
         <x:v>Canada</x:v>
       </x:c>
@@ -2302,12 +2363,14 @@
         <x:v>Canada</x:v>
       </x:c>
       <x:c r="N38" s="2" t="str">
-        <x:v>Verified city - street address pending</x:v>
+        <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O38" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/</x:v>
-      </x:c>
-      <x:c r="P38" s="2"/>
+        <x:v>https://www.molsoncoors.com/our-locations/ca/brewery/stjohn</x:v>
+      </x:c>
+      <x:c r="P38" s="2" t="str">
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="30" hidden="1">
       <x:c r="A39" s="2" t="str">
@@ -11596,7 +11659,7 @@
         <x:v>Molson Coors Beverage Company</x:v>
       </x:c>
       <x:c r="D235" s="2" t="str">
-        <x:v>Molson Coors - Toronto</x:v>
+        <x:v>Molson Coors - Toronto Brewery</x:v>
       </x:c>
       <x:c r="E235" s="2" t="str">
         <x:v>Brewery</x:v>
@@ -11629,10 +11692,10 @@
         <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O235" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/ca/our-locations</x:v>
+        <x:v>https://www.molsoncoors.com/our-locations/ca/brewery/toronto</x:v>
       </x:c>
       <x:c r="P235" s="2" t="str">
-        <x:v>Current Canadian brewery; exact address published by Molson Coors.</x:v>
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
       </x:c>
     </x:row>
     <x:row r="236" ht="30" hidden="1">
@@ -11646,7 +11709,7 @@
         <x:v>Molson Coors Beverage Company</x:v>
       </x:c>
       <x:c r="D236" s="2" t="str">
-        <x:v>Molson Coors - Moncton</x:v>
+        <x:v>Molson Coors - Moncton Brewery</x:v>
       </x:c>
       <x:c r="E236" s="2" t="str">
         <x:v>Brewery</x:v>
@@ -11679,10 +11742,10 @@
         <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O236" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/ca/our-locations</x:v>
+        <x:v>https://www.molsoncoors.com/our-locations/ca/brewery/moncton</x:v>
       </x:c>
       <x:c r="P236" s="2" t="str">
-        <x:v>Current Canadian brewery; exact address published by Molson Coors.</x:v>
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
       </x:c>
     </x:row>
     <x:row r="237" ht="30" hidden="1">
@@ -11701,14 +11764,18 @@
       <x:c r="E237" s="2" t="str">
         <x:v>Craft brewery</x:v>
       </x:c>
-      <x:c r="F237" s="2"/>
+      <x:c r="F237" s="2" t="str">
+        <x:v>1485 Rue Ottawa</x:v>
+      </x:c>
       <x:c r="G237" s="2" t="str">
-        <x:v>Montreal</x:v>
+        <x:v>Montréal</x:v>
       </x:c>
       <x:c r="H237" s="2" t="str">
         <x:v>QC</x:v>
       </x:c>
-      <x:c r="I237" s="2"/>
+      <x:c r="I237" s="2" t="str">
+        <x:v>H3C 1S9</x:v>
+      </x:c>
       <x:c r="J237" s="2" t="str">
         <x:v>Canada</x:v>
       </x:c>
@@ -11722,13 +11789,13 @@
         <x:v>Canada</x:v>
       </x:c>
       <x:c r="N237" s="2" t="str">
-        <x:v>Verified city - official source</x:v>
+        <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O237" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/ca/our-locations</x:v>
+        <x:v>https://www.molsoncoors.com/our-locations/ca/brewery/brasseur-de-montreal</x:v>
       </x:c>
       <x:c r="P237" s="2" t="str">
-        <x:v>Listed in Molson Coors' current Americas brewery network.</x:v>
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
       </x:c>
     </x:row>
     <x:row r="238" ht="30" hidden="1">
@@ -11747,14 +11814,18 @@
       <x:c r="E238" s="2" t="str">
         <x:v>Craft brewery</x:v>
       </x:c>
-      <x:c r="F238" s="2"/>
+      <x:c r="F238" s="2" t="str">
+        <x:v>139 Mill Street</x:v>
+      </x:c>
       <x:c r="G238" s="2" t="str">
         <x:v>Creemore</x:v>
       </x:c>
       <x:c r="H238" s="2" t="str">
         <x:v>ON</x:v>
       </x:c>
-      <x:c r="I238" s="2"/>
+      <x:c r="I238" s="2" t="str">
+        <x:v>L0M 1G0</x:v>
+      </x:c>
       <x:c r="J238" s="2" t="str">
         <x:v>Canada</x:v>
       </x:c>
@@ -11768,13 +11839,13 @@
         <x:v>Canada</x:v>
       </x:c>
       <x:c r="N238" s="2" t="str">
-        <x:v>Verified city - official source</x:v>
+        <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O238" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/ca/our-locations</x:v>
+        <x:v>https://www.molsoncoors.com/our-locations/ca/brewery/creemore-springs</x:v>
       </x:c>
       <x:c r="P238" s="2" t="str">
-        <x:v>Listed in Molson Coors' current Americas brewery network.</x:v>
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
       </x:c>
     </x:row>
     <x:row r="239" ht="30" hidden="1">
@@ -11793,14 +11864,18 @@
       <x:c r="E239" s="2" t="str">
         <x:v>Craft brewery</x:v>
       </x:c>
-      <x:c r="F239" s="2"/>
+      <x:c r="F239" s="2" t="str">
+        <x:v>1441 Cartwright Street</x:v>
+      </x:c>
       <x:c r="G239" s="2" t="str">
         <x:v>Vancouver</x:v>
       </x:c>
       <x:c r="H239" s="2" t="str">
         <x:v>BC</x:v>
       </x:c>
-      <x:c r="I239" s="2"/>
+      <x:c r="I239" s="2" t="str">
+        <x:v>V6H 3R7</x:v>
+      </x:c>
       <x:c r="J239" s="2" t="str">
         <x:v>Canada</x:v>
       </x:c>
@@ -11814,13 +11889,13 @@
         <x:v>Canada</x:v>
       </x:c>
       <x:c r="N239" s="2" t="str">
-        <x:v>Verified city - official source</x:v>
+        <x:v>Verified - official source</x:v>
       </x:c>
       <x:c r="O239" s="2" t="str">
-        <x:v>https://www.molsoncoors.com/ca/our-locations</x:v>
+        <x:v>https://www.molsoncoors.com/our-locations/ca/brewery/granville-island</x:v>
       </x:c>
       <x:c r="P239" s="2" t="str">
-        <x:v>Listed in Molson Coors' current Americas brewery network.</x:v>
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
       </x:c>
     </x:row>
     <x:row r="240" ht="30" hidden="1">
@@ -11840,7 +11915,7 @@
         <x:v>Craft brewery</x:v>
       </x:c>
       <x:c r="F240" s="2" t="str">
-        <x:v>1250 Avenue de la Station</x:v>
+        <x:v>1250 Avenue De La Station</x:v>
       </x:c>
       <x:c r="G240" s="2" t="str">
         <x:v>Shawinigan</x:v>
@@ -11870,7 +11945,7 @@
         <x:v>https://www.molsoncoors.com/our-locations/ca/brewery/le-trou-du-diable</x:v>
       </x:c>
       <x:c r="P240" s="2" t="str">
-        <x:v>Exact address published by Molson Coors.</x:v>
+        <x:v>Current facility verified in Molson Coors' official Americas brewery directory during the 2026-08-17 nationwide/state-by-state audit. Official street address added; no new coordinate was invented.</x:v>
       </x:c>
     </x:row>
     <x:row r="241" ht="30" hidden="1">
@@ -19039,6 +19114,852 @@
       </x:c>
       <x:c r="P388" t="str">
         <x:v>Clif Bar Baking Company production location reconciled against current company, career, directory, and regulatory evidence. Coordinates are the GeoNames city centroid; replace with exact plant coordinates when verified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="389">
+      <x:c r="A389" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B389" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C389" t="str">
+        <x:v>Elysian Brewing</x:v>
+      </x:c>
+      <x:c r="D389" t="str">
+        <x:v>Elysian - Capitol Hill Brewery</x:v>
+      </x:c>
+      <x:c r="E389" t="str">
+        <x:v>Craft brewery</x:v>
+      </x:c>
+      <x:c r="F389" t="str">
+        <x:v>1221 E Pike St</x:v>
+      </x:c>
+      <x:c r="G389" t="str">
+        <x:v>Seattle</x:v>
+      </x:c>
+      <x:c r="H389" t="str">
+        <x:v>WA</x:v>
+      </x:c>
+      <x:c r="I389" t="str">
+        <x:v>98122</x:v>
+      </x:c>
+      <x:c r="J389" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K389" t="n">
+        <x:v>47.60621</x:v>
+      </x:c>
+      <x:c r="L389" t="n">
+        <x:v>-122.33207</x:v>
+      </x:c>
+      <x:c r="M389" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N389" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O389" t="str">
+        <x:v>https://www.elysianbrewing.com/node/939</x:v>
+      </x:c>
+      <x:c r="P389" t="str">
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="390">
+      <x:c r="A390" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B390" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C390" t="str">
+        <x:v>Wicked Weed Brewing</x:v>
+      </x:c>
+      <x:c r="D390" t="str">
+        <x:v>Wicked Weed - Original Brewpub Brewery</x:v>
+      </x:c>
+      <x:c r="E390" t="str">
+        <x:v>Craft brewery</x:v>
+      </x:c>
+      <x:c r="F390" t="str">
+        <x:v>91 Biltmore Ave</x:v>
+      </x:c>
+      <x:c r="G390" t="str">
+        <x:v>Asheville</x:v>
+      </x:c>
+      <x:c r="H390" t="str">
+        <x:v>NC</x:v>
+      </x:c>
+      <x:c r="I390" t="str">
+        <x:v>28801</x:v>
+      </x:c>
+      <x:c r="J390" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K390" t="n">
+        <x:v>35.60095</x:v>
+      </x:c>
+      <x:c r="L390" t="n">
+        <x:v>-82.55402</x:v>
+      </x:c>
+      <x:c r="M390" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N390" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O390" t="str">
+        <x:v>https://www.wickedweedbrewing.com/</x:v>
+      </x:c>
+      <x:c r="P390" t="str">
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="391">
+      <x:c r="A391" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B391" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C391" t="str">
+        <x:v>Wicked Weed Brewing</x:v>
+      </x:c>
+      <x:c r="D391" t="str">
+        <x:v>Wicked Weed - Funkatorium</x:v>
+      </x:c>
+      <x:c r="E391" t="str">
+        <x:v>Sour craft brewery</x:v>
+      </x:c>
+      <x:c r="F391" t="str">
+        <x:v>147 Coxe Ave</x:v>
+      </x:c>
+      <x:c r="G391" t="str">
+        <x:v>Asheville</x:v>
+      </x:c>
+      <x:c r="H391" t="str">
+        <x:v>NC</x:v>
+      </x:c>
+      <x:c r="I391" t="str">
+        <x:v>28801</x:v>
+      </x:c>
+      <x:c r="J391" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K391" t="n">
+        <x:v>35.60095</x:v>
+      </x:c>
+      <x:c r="L391" t="n">
+        <x:v>-82.55402</x:v>
+      </x:c>
+      <x:c r="M391" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N391" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O391" t="str">
+        <x:v>https://www.wickedweedbrewing.com/location/funkatorium/</x:v>
+      </x:c>
+      <x:c r="P391" t="str">
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="392">
+      <x:c r="A392" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B392" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C392" t="str">
+        <x:v>Wicked Weed Brewing</x:v>
+      </x:c>
+      <x:c r="D392" t="str">
+        <x:v>Wicked Weed West Production Brewery</x:v>
+      </x:c>
+      <x:c r="E392" t="str">
+        <x:v>Craft production brewery</x:v>
+      </x:c>
+      <x:c r="F392" t="str">
+        <x:v>145 Jacob Holm Way</x:v>
+      </x:c>
+      <x:c r="G392" t="str">
+        <x:v>Candler</x:v>
+      </x:c>
+      <x:c r="H392" t="str">
+        <x:v>NC</x:v>
+      </x:c>
+      <x:c r="I392" t="str">
+        <x:v>28715</x:v>
+      </x:c>
+      <x:c r="J392" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K392" t="n">
+        <x:v>35.5365</x:v>
+      </x:c>
+      <x:c r="L392" t="n">
+        <x:v>-82.69291</x:v>
+      </x:c>
+      <x:c r="M392" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N392" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O392" t="str">
+        <x:v>https://www.wickedweedbrewing.com/location/wicked-weed-west/</x:v>
+      </x:c>
+      <x:c r="P392" t="str">
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="393">
+      <x:c r="A393" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B393" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C393" t="str">
+        <x:v>Karbach Brewing Co</x:v>
+      </x:c>
+      <x:c r="D393" t="str">
+        <x:v>Karbach Brewery</x:v>
+      </x:c>
+      <x:c r="E393" t="str">
+        <x:v>Craft brewery</x:v>
+      </x:c>
+      <x:c r="F393" t="str">
+        <x:v>2032 Karbach Street</x:v>
+      </x:c>
+      <x:c r="G393" t="str">
+        <x:v>Houston</x:v>
+      </x:c>
+      <x:c r="H393" t="str">
+        <x:v>TX</x:v>
+      </x:c>
+      <x:c r="I393" t="str">
+        <x:v>77092</x:v>
+      </x:c>
+      <x:c r="J393" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K393" t="n">
+        <x:v>29.76328</x:v>
+      </x:c>
+      <x:c r="L393" t="n">
+        <x:v>-95.36327</x:v>
+      </x:c>
+      <x:c r="M393" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="N393" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O393" t="str">
+        <x:v>https://www.karbachbrewing.com/brewery/</x:v>
+      </x:c>
+      <x:c r="P393" t="str">
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="394">
+      <x:c r="A394" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B394" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C394" t="str">
+        <x:v>Devils Backbone Brewing Co</x:v>
+      </x:c>
+      <x:c r="D394" t="str">
+        <x:v>Devils Backbone - Basecamp Brewery</x:v>
+      </x:c>
+      <x:c r="E394" t="str">
+        <x:v>Craft brewery / distillery</x:v>
+      </x:c>
+      <x:c r="F394" t="str">
+        <x:v>200 Crandall Run</x:v>
+      </x:c>
+      <x:c r="G394" t="str">
+        <x:v>Roseland</x:v>
+      </x:c>
+      <x:c r="H394" t="str">
+        <x:v>VA</x:v>
+      </x:c>
+      <x:c r="I394" t="str">
+        <x:v>22967</x:v>
+      </x:c>
+      <x:c r="J394" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K394" t="n">
+        <x:v>37.74764</x:v>
+      </x:c>
+      <x:c r="L394" t="n">
+        <x:v>-78.97586</x:v>
+      </x:c>
+      <x:c r="M394" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="N394" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O394" t="str">
+        <x:v>https://www.dbbrewingcompany.com/contact-us/</x:v>
+      </x:c>
+      <x:c r="P394" t="str">
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="395">
+      <x:c r="A395" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B395" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C395" t="str">
+        <x:v>Devils Backbone Brewing Co</x:v>
+      </x:c>
+      <x:c r="D395" t="str">
+        <x:v>Devils Backbone - Outpost Production Brewery</x:v>
+      </x:c>
+      <x:c r="E395" t="str">
+        <x:v>Craft production brewery</x:v>
+      </x:c>
+      <x:c r="F395" t="str">
+        <x:v>50 Northwind Lane</x:v>
+      </x:c>
+      <x:c r="G395" t="str">
+        <x:v>Lexington</x:v>
+      </x:c>
+      <x:c r="H395" t="str">
+        <x:v>VA</x:v>
+      </x:c>
+      <x:c r="I395" t="str">
+        <x:v>24450</x:v>
+      </x:c>
+      <x:c r="J395" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K395" t="n">
+        <x:v>37.78402</x:v>
+      </x:c>
+      <x:c r="L395" t="n">
+        <x:v>-79.44282</x:v>
+      </x:c>
+      <x:c r="M395" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="N395" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O395" t="str">
+        <x:v>https://www.dbbrewingcompany.com/location/outpost/</x:v>
+      </x:c>
+      <x:c r="P395" t="str">
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="396">
+      <x:c r="A396" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B396" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C396" t="str">
+        <x:v>Four Peaks Brewing Co</x:v>
+      </x:c>
+      <x:c r="D396" t="str">
+        <x:v>Four Peaks - 8th Street Brewery</x:v>
+      </x:c>
+      <x:c r="E396" t="str">
+        <x:v>Craft brewery</x:v>
+      </x:c>
+      <x:c r="F396" t="str">
+        <x:v>1340 E 8th St #104</x:v>
+      </x:c>
+      <x:c r="G396" t="str">
+        <x:v>Tempe</x:v>
+      </x:c>
+      <x:c r="H396" t="str">
+        <x:v>AZ</x:v>
+      </x:c>
+      <x:c r="I396" t="str">
+        <x:v>85281</x:v>
+      </x:c>
+      <x:c r="J396" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K396" t="n">
+        <x:v>33.41477</x:v>
+      </x:c>
+      <x:c r="L396" t="n">
+        <x:v>-111.90931</x:v>
+      </x:c>
+      <x:c r="M396" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N396" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O396" t="str">
+        <x:v>https://www.fourpeaks.com/8th-street-pub</x:v>
+      </x:c>
+      <x:c r="P396" t="str">
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="397">
+      <x:c r="A397" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B397" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C397" t="str">
+        <x:v>Four Peaks Brewing Co</x:v>
+      </x:c>
+      <x:c r="D397" t="str">
+        <x:v>Four Peaks - Wilson Production Brewery</x:v>
+      </x:c>
+      <x:c r="E397" t="str">
+        <x:v>Craft production brewery</x:v>
+      </x:c>
+      <x:c r="F397" t="str">
+        <x:v>2401 S Wilson St</x:v>
+      </x:c>
+      <x:c r="G397" t="str">
+        <x:v>Tempe</x:v>
+      </x:c>
+      <x:c r="H397" t="str">
+        <x:v>AZ</x:v>
+      </x:c>
+      <x:c r="I397" t="str">
+        <x:v>85282</x:v>
+      </x:c>
+      <x:c r="J397" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K397" t="n">
+        <x:v>33.41477</x:v>
+      </x:c>
+      <x:c r="L397" t="n">
+        <x:v>-111.90931</x:v>
+      </x:c>
+      <x:c r="M397" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N397" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O397" t="str">
+        <x:v>https://www.fourpeaks.com/wilson-tasting-room-event-space</x:v>
+      </x:c>
+      <x:c r="P397" t="str">
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="398">
+      <x:c r="A398" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B398" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C398" t="str">
+        <x:v>Cisco Brewers</x:v>
+      </x:c>
+      <x:c r="D398" t="str">
+        <x:v>Cisco Brewers - Nantucket Brewery</x:v>
+      </x:c>
+      <x:c r="E398" t="str">
+        <x:v>Craft brewery / distillery / winery</x:v>
+      </x:c>
+      <x:c r="F398" t="str">
+        <x:v>5 Bartlett Farm Rd</x:v>
+      </x:c>
+      <x:c r="G398" t="str">
+        <x:v>Nantucket</x:v>
+      </x:c>
+      <x:c r="H398" t="str">
+        <x:v>MA</x:v>
+      </x:c>
+      <x:c r="I398" t="str">
+        <x:v>02554</x:v>
+      </x:c>
+      <x:c r="J398" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K398" t="n">
+        <x:v>41.28346</x:v>
+      </x:c>
+      <x:c r="L398" t="n">
+        <x:v>-70.09946</x:v>
+      </x:c>
+      <x:c r="M398" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="N398" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O398" t="str">
+        <x:v>https://www.ciscobrewers.com/nantucket</x:v>
+      </x:c>
+      <x:c r="P398" t="str">
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="399">
+      <x:c r="A399" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B399" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C399" t="str">
+        <x:v>La Rubia Beer</x:v>
+      </x:c>
+      <x:c r="D399" t="str">
+        <x:v>Casa La Rubia Brewery</x:v>
+      </x:c>
+      <x:c r="E399" t="str">
+        <x:v>Craft brewery</x:v>
+      </x:c>
+      <x:c r="F399" t="str">
+        <x:v>55 NW 25th St</x:v>
+      </x:c>
+      <x:c r="G399" t="str">
+        <x:v>Miami</x:v>
+      </x:c>
+      <x:c r="H399" t="str">
+        <x:v>FL</x:v>
+      </x:c>
+      <x:c r="I399" t="str">
+        <x:v>33127</x:v>
+      </x:c>
+      <x:c r="J399" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K399" t="n">
+        <x:v>25.77427</x:v>
+      </x:c>
+      <x:c r="L399" t="n">
+        <x:v>-80.19366</x:v>
+      </x:c>
+      <x:c r="M399" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N399" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O399" t="str">
+        <x:v>https://www.larubia.beer/faq</x:v>
+      </x:c>
+      <x:c r="P399" t="str">
+        <x:v>Facility and ownership verified during the 2026-08-17 national Anheuser-Busch audit. Current A-B craft portfolio source: https://www.anheuser-busch.com/newsroom/CraftMomentum.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="400">
+      <x:c r="A400" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B400" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C400" t="str">
+        <x:v>Busch Agricultural Resources</x:v>
+      </x:c>
+      <x:c r="D400" t="str">
+        <x:v>Idaho Falls Barley Elevator</x:v>
+      </x:c>
+      <x:c r="E400" t="str">
+        <x:v>Barley elevator</x:v>
+      </x:c>
+      <x:c r="F400" t="str">
+        <x:v>2121 West 145 North</x:v>
+      </x:c>
+      <x:c r="G400" t="str">
+        <x:v>Idaho Falls</x:v>
+      </x:c>
+      <x:c r="H400" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="I400" t="str">
+        <x:v>83402</x:v>
+      </x:c>
+      <x:c r="J400" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K400" t="n">
+        <x:v>43.46658</x:v>
+      </x:c>
+      <x:c r="L400" t="n">
+        <x:v>-112.03414</x:v>
+      </x:c>
+      <x:c r="M400" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N400" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O400" t="str">
+        <x:v>https://www.anheuser-busch.com/newsroom/Anheuser-Busch-to-Sponsor-Idaho-Honor-Flights-Inaugural-Mission-to-Washington-DC-This-September</x:v>
+      </x:c>
+      <x:c r="P400" t="str">
+        <x:v>Current A-B source confirms five Idaho agricultural facilities; 2026 local facility tour identifies this elevator and street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="401">
+      <x:c r="A401" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B401" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C401" t="str">
+        <x:v>Busch Agricultural Resources</x:v>
+      </x:c>
+      <x:c r="D401" t="str">
+        <x:v>Idaho Falls Malt Plant - Yellowstone Highway</x:v>
+      </x:c>
+      <x:c r="E401" t="str">
+        <x:v>Malt plant</x:v>
+      </x:c>
+      <x:c r="F401" t="str">
+        <x:v>5755 South Yellowstone Highway</x:v>
+      </x:c>
+      <x:c r="G401" t="str">
+        <x:v>Idaho Falls</x:v>
+      </x:c>
+      <x:c r="H401" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="I401" t="str">
+        <x:v>83402</x:v>
+      </x:c>
+      <x:c r="J401" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K401" t="n">
+        <x:v>43.46658</x:v>
+      </x:c>
+      <x:c r="L401" t="n">
+        <x:v>-112.03414</x:v>
+      </x:c>
+      <x:c r="M401" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N401" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O401" t="str">
+        <x:v>https://www.anheuser-busch.com/newsroom/Anheuser-Busch-to-Sponsor-Idaho-Honor-Flights-Inaugural-Mission-to-Washington-DC-This-September</x:v>
+      </x:c>
+      <x:c r="P401" t="str">
+        <x:v>Current A-B source confirms the Idaho Falls malt operation; 2026 local facility tour provides this street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="402">
+      <x:c r="A402" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B402" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C402" t="str">
+        <x:v>Busch Agricultural Resources</x:v>
+      </x:c>
+      <x:c r="D402" t="str">
+        <x:v>Idaho Falls Malt Plant - InteGrow</x:v>
+      </x:c>
+      <x:c r="E402" t="str">
+        <x:v>Malt plant</x:v>
+      </x:c>
+      <x:c r="F402" t="str">
+        <x:v>5005 South 15th West</x:v>
+      </x:c>
+      <x:c r="G402" t="str">
+        <x:v>Idaho Falls</x:v>
+      </x:c>
+      <x:c r="H402" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="I402" t="str">
+        <x:v>83402</x:v>
+      </x:c>
+      <x:c r="J402" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K402" t="n">
+        <x:v>43.46658</x:v>
+      </x:c>
+      <x:c r="L402" t="n">
+        <x:v>-112.03414</x:v>
+      </x:c>
+      <x:c r="M402" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N402" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O402" t="str">
+        <x:v>https://www.anheuser-busch.com/agriculture</x:v>
+      </x:c>
+      <x:c r="P402" t="str">
+        <x:v>A-B reports 11 major U.S. agriculture facilities; 2026 Idaho reporting confirms two active Idaho Falls malt plants. Address corroborated by Idaho Barley Commission materials.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="403">
+      <x:c r="A403" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B403" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C403" t="str">
+        <x:v>Busch Agricultural Resources</x:v>
+      </x:c>
+      <x:c r="D403" t="str">
+        <x:v>Idaho Falls Seed Facility</x:v>
+      </x:c>
+      <x:c r="E403" t="str">
+        <x:v>Barley seed facility</x:v>
+      </x:c>
+      <x:c r="F403"/>
+      <x:c r="G403" t="str">
+        <x:v>Idaho Falls</x:v>
+      </x:c>
+      <x:c r="H403" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="I403"/>
+      <x:c r="J403" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K403" t="n">
+        <x:v>43.46658</x:v>
+      </x:c>
+      <x:c r="L403" t="n">
+        <x:v>-112.03414</x:v>
+      </x:c>
+      <x:c r="M403" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N403" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O403" t="str">
+        <x:v>https://www.anheuser-busch.com/newsroom/Anheuser-Busch-to-Sponsor-Idaho-Honor-Flights-Inaugural-Mission-to-Washington-DC-This-September</x:v>
+      </x:c>
+      <x:c r="P403" t="str">
+        <x:v>Current A-B source confirms five Idaho agricultural facilities; 2026 local reporting identifies the Idaho Falls seed facility. Street address remains pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="404">
+      <x:c r="A404" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B404" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C404" t="str">
+        <x:v>Busch Agricultural Resources</x:v>
+      </x:c>
+      <x:c r="D404" t="str">
+        <x:v>Elk Mountain Farms</x:v>
+      </x:c>
+      <x:c r="E404" t="str">
+        <x:v>Hop farm</x:v>
+      </x:c>
+      <x:c r="F404" t="str">
+        <x:v>822 Budweiser Loop</x:v>
+      </x:c>
+      <x:c r="G404" t="str">
+        <x:v>Bonners Ferry</x:v>
+      </x:c>
+      <x:c r="H404" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="I404" t="str">
+        <x:v>83805</x:v>
+      </x:c>
+      <x:c r="J404" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K404" t="n">
+        <x:v>48.69133</x:v>
+      </x:c>
+      <x:c r="L404" t="n">
+        <x:v>-116.31631</x:v>
+      </x:c>
+      <x:c r="M404" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N404" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O404" t="str">
+        <x:v>https://www.anheuser-busch.com/agriculture</x:v>
+      </x:c>
+      <x:c r="P404" t="str">
+        <x:v>Elk Mountain Farms is the fifth current Idaho agricultural facility; ownership and operation are corroborated by University of Idaho research reporting.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="405">
+      <x:c r="A405" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B405" t="str">
+        <x:v>AB InBev Belgium N.V. (HQ)</x:v>
+      </x:c>
+      <x:c r="C405" t="str">
+        <x:v>Busch Agricultural Resources</x:v>
+      </x:c>
+      <x:c r="D405" t="str">
+        <x:v>Jonesboro Rice Mill</x:v>
+      </x:c>
+      <x:c r="E405" t="str">
+        <x:v>Rice mill</x:v>
+      </x:c>
+      <x:c r="F405" t="str">
+        <x:v>3723 County Road 905</x:v>
+      </x:c>
+      <x:c r="G405" t="str">
+        <x:v>Jonesboro</x:v>
+      </x:c>
+      <x:c r="H405" t="str">
+        <x:v>AR</x:v>
+      </x:c>
+      <x:c r="I405" t="str">
+        <x:v>72401</x:v>
+      </x:c>
+      <x:c r="J405" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K405" t="n">
+        <x:v>35.874178</x:v>
+      </x:c>
+      <x:c r="L405" t="n">
+        <x:v>-90.601151</x:v>
+      </x:c>
+      <x:c r="M405" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="N405" t="str">
+        <x:v>Verified - source-supported</x:v>
+      </x:c>
+      <x:c r="O405" t="str">
+        <x:v>https://www.anheuser-busch.com/about/brewing-process</x:v>
+      </x:c>
+      <x:c r="P405" t="str">
+        <x:v>Current A-B brewing page confirms the Jonesboro rice mill; Arkansas DEQ provides the street address and postprocessed facility GPS coordinate.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -19052,7 +19973,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f8837b2f5924a3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cfd8648d2684e89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19136,16 +20057,16 @@
         <x:v>AB InBev Belgium N.V. (HQ)</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Added Grupo Modelo's eight official industrial breweries in Mexico.</x:v>
+        <x:v>Nationwide production audit: 9 current large U.S. breweries, 14 current/source-supported owned craft brewery facilities, 6 specifically identified agricultural production sites, plus 8 Grupo Modelo breweries in Mexico.</x:v>
       </x:c>
       <x:c r="D4" t="n">
-        <x:v>8</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="E4" t="n">
-        <x:v>8</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>Mexico brewery network added from Grupo Modelo official sources.</x:v>
+        <x:v>AB InBev account now contains 37 mapped production/agriculture sites. Three announced 2026 closures (Fairfield, Merrimack, Newark) were replaced. A-B reports 11 major U.S. agriculture facilities; five not publicly enumerated remain unresolved rather than guessed.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -19156,16 +20077,16 @@
         <x:v>Molson Coors Beverage Company</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Added six missing Canadian primary/craft breweries.</x:v>
+        <x:v>Nationwide U.S. state-by-state and Canadian province audit reconciled to Molson Coors' current official Americas directory: 6 U.S. large breweries, 5 Canadian large breweries, and 4 Canadian craft breweries.</x:v>
       </x:c>
       <x:c r="D5" t="n">
-        <x:v>6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:v>3</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>Current official Americas brewery network reconciled.</x:v>
+        <x:v>All 15 current official North American brewery listings are captured with Molson Coors-published street addresses. Closed/divested legacy U.S. sites are excluded.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -19348,10 +20269,30 @@
         <x:v>Fair Lawn is excluded as closed; all six current bakery plants are mapped with street addresses.</x:v>
       </x:c>
     </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>Brewing</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>Metal Container Corporation</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Retained as a separate strategic account: five can plants (Arnold, Jacksonville, Mira Loma, Newburgh, Windsor) and two lid plants (Oklahoma City, Riverside).</x:v>
+      </x:c>
+      <x:c r="D15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>Seven MCC locations retained separately. Arnold and Jacksonville are corroborated by current 2026 A-B announcements; the other five retain official network support but need fresh plant-specific confirmation.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cbb79c8541446c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2287b0ba27b646c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19383,20 +20324,20 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
-        <x:v>Added verified or source-supported manufacturing, bottling, brewing, packaging, and bakery facilities across the United States, Canada, and Mexico, including nationwide Coca-Cola, Grupo Bimbo, Aspire Bakeries, and Mondelez audits; ordinary distribution-only sites remain excluded.</x:v>
+        <x:v>Added verified or source-supported manufacturing, bottling, brewing, packaging, bakery, and agricultural production facilities across the United States, Canada, and Mexico, including national Coca-Cola, Grupo Bimbo, Aspire Bakeries, Mondelez, Molson Coors, and Anheuser-Busch audits; ordinary distribution-only sites remain excluded.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15">
       <x:c r="A4" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="s">
-        <x:v>14</x:v>
+      <x:c r="B4" s="2" t="str">
+        <x:v>Operating / Bottler Entity separates the strategic parent from the actual company operating each production facility.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30">
       <x:c r="A5" s="2" t="s">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B5" s="2" t="str">
         <x:v>Completed a nationwide U.S. Coca-Cola production audit across the major bottling systems and confirmed regional producers. Current official sources are preferred; entries supported only at city level are explicitly flagged.</x:v>
@@ -19404,15 +20345,15 @@
     </x:row>
     <x:row r="6" ht="30">
       <x:c r="A6" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="s">
         <x:v>16</x:v>
-      </x:c>
-      <x:c r="B6" s="2" t="s">
-        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30">
       <x:c r="A7" s="2" t="s">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B7" s="2" t="str">
         <x:v>Manufacturing, packaging, bottling, processing, breweries, and sites with meaningful production/material-handling systems. Distribution-only branches are excluded unless production is explicitly documented.</x:v>
@@ -19420,7 +20361,7 @@
     </x:row>
     <x:row r="8" ht="30">
       <x:c r="A8" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B8" s="2" t="str">
         <x:v>Official company pages and current regulatory filings preferred. Exact street addresses are used only when published; city-only rows are flagged, and their coordinates are city-centroid estimates for mapping continuity.</x:v>
@@ -19428,7 +20369,7 @@
     </x:row>
     <x:row r="9" ht="30">
       <x:c r="A9" s="2" t="s">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B9" s="2" t="str">
         <x:v>Street addresses are recorded where company, directory, or regulatory sources publish them. Map coordinates remain transparent GeoNames city centroids until exact facility coordinates are independently verified.</x:v>
@@ -19784,7 +20725,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>Anheuser-Busch Brewery - Fairfield</x:v>
+        <x:v>Goose Island - Fulton Street Brewery</x:v>
       </x:c>
       <x:c r="C17" s="22" t="str">
         <x:v>Added — approximate</x:v>
@@ -19796,7 +20737,7 @@
         <x:v>City-center fallback</x:v>
       </x:c>
       <x:c r="F17" s="23" t="str">
-        <x:v>Fairfield, California; GeoNames ID 5347335</x:v>
+        <x:v>Chicago, IL; GeoNames ID 4887398; exact facility coordinate should replace this point when verified</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="28">
@@ -19804,7 +20745,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B18" s="22" t="str">
-        <x:v>Anheuser-Busch Brewery - Merrimack</x:v>
+        <x:v>Golden Road - Atwater Village Brewery</x:v>
       </x:c>
       <x:c r="C18" s="22" t="str">
         <x:v>Added — approximate</x:v>
@@ -19816,7 +20757,7 @@
         <x:v>City-center fallback</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>Merrimack, New Hampshire; GeoNames ID 5089478</x:v>
+        <x:v>Los Angeles, CA; GeoNames ID 5368361; exact facility coordinate should replace this point when verified</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="28">
@@ -19824,7 +20765,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B19" s="22" t="str">
-        <x:v>Anheuser-Busch Brewery - Newark</x:v>
+        <x:v>Golden Road - Anaheim Brewery</x:v>
       </x:c>
       <x:c r="C19" s="22" t="str">
         <x:v>Added — approximate</x:v>
@@ -19836,7 +20777,7 @@
         <x:v>City-center fallback</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>Newark, New Jersey; GeoNames ID 5101798</x:v>
+        <x:v>Anaheim, CA; GeoNames ID 5323810; exact facility coordinate should replace this point when verified</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="28">
@@ -20050,13 +20991,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D30" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E30" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F30" s="23" t="str">
-        <x:v>Golden, Colorado; GeoNames ID 5423294</x:v>
+        <x:v>12th &amp; Ford Street, Golden, CO 80401; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="28">
@@ -20070,13 +21011,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D31" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E31" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F31" s="23" t="str">
-        <x:v>Milwaukee, Wisconsin; GeoNames ID 5263045</x:v>
+        <x:v>4000 W. State Street, Milwaukee, WI 53208; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="28">
@@ -20090,13 +21031,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D32" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E32" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>Albany, Georgia; GeoNames ID 4179320</x:v>
+        <x:v>405 Cordele Road, Albany, GA 31705; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="28">
@@ -20110,13 +21051,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D33" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E33" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F33" s="23" t="str">
-        <x:v>Fort Worth, Texas; GeoNames ID 4691930</x:v>
+        <x:v>7001 South Freeway, Fort Worth, TX 76134; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="28">
@@ -20130,13 +21071,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D34" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E34" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F34" s="23" t="str">
-        <x:v>Trenton, Ohio; GeoNames ID 4526469</x:v>
+        <x:v>2525 Wayne Madison Rd., Trenton, OH 45067; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="28">
@@ -20150,13 +21091,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D35" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E35" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F35" s="23" t="str">
-        <x:v>Elkton, Virginia; GeoNames ID 4757467</x:v>
+        <x:v>5135 S. East Side Highway, Elkton, VA 22827; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="28">
@@ -20170,13 +21111,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D36" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E36" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>Chilliwack, British Columbia; GeoNames ID 5921356</x:v>
+        <x:v>45620 Kerr Avenue, Chilliwack, BC V2R 0Z7; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="28">
@@ -20190,13 +21131,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D37" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E37" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F37" s="23" t="str">
-        <x:v>Longueuil, Quebec; GeoNames ID 6059891</x:v>
+        <x:v>6125 Route De L'aeroport, Saint-Hubert, QC J3Y 8Y9; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="28">
@@ -20210,13 +21151,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D38" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E38" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F38" s="23" t="str">
-        <x:v>St. John's, Newfoundland and Labrador; GeoNames ID 6324733</x:v>
+        <x:v>131 Circular Road, St. John's, NL A1C 5W1; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="28">
@@ -23667,16 +24608,16 @@
         <x:v>Indianapolis Manufacturing Facility</x:v>
       </x:c>
       <x:c r="C211" s="22" t="str">
-        <x:v>Added</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D211" s="22" t="str">
-        <x:v>U.S. Census Geocoder, benchmark 4</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E211" s="22" t="str">
-        <x:v>Exact address match</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F211" s="23" t="str">
-        <x:v>5000 W 25TH ST, INDIANAPOLIS, IN, 46224</x:v>
+        <x:v>1 Carlingview Drive, Toronto, ON M9W 5E5; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="212" ht="28">
@@ -23690,13 +24631,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D212" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E212" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F212" s="23" t="str">
-        <x:v>Roanoke, Virginia; GeoNames ID 4782167; replaces stale Portland entry</x:v>
+        <x:v>170 Macnaughton Avenue, Moncton, NB E1H 3L9; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="213">
@@ -23710,13 +24651,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D213" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E213" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F213" s="23" t="str">
-        <x:v>Cincinnati, Ohio; GeoNames ID 4508722</x:v>
+        <x:v>1485 Rue Ottawa, Montréal, QC H3C 1S9; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="214">
@@ -23727,16 +24668,16 @@
         <x:v>Twinsburg Manufacturing Facility</x:v>
       </x:c>
       <x:c r="C214" s="22" t="str">
-        <x:v>Added</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D214" s="22" t="str">
-        <x:v>U.S. Census Geocoder, benchmark 4</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E214" s="22" t="str">
-        <x:v>Exact address match</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F214" s="23" t="str">
-        <x:v>1882 HIGHLAND RD, TWINSBURG, OH, 44087</x:v>
+        <x:v>139 Mill Street, Creemore, ON L0M 1G0; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="215">
@@ -23750,13 +24691,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D215" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E215" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F215" s="23" t="str">
-        <x:v>West Memphis, Arkansas; GeoNames ID 4135865</x:v>
+        <x:v>1441 Cartwright Street, Vancouver, BC V6H 3R7; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="216" ht="28">
@@ -23770,13 +24711,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D216" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Existing mapped coordinate; official street address verified by Molson Coors</x:v>
       </x:c>
       <x:c r="E216" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Approximate / existing point</x:v>
       </x:c>
       <x:c r="F216" s="23" t="str">
-        <x:v>Nashville, Tennessee; GeoNames ID 4644585; replaces stale Memphis entry</x:v>
+        <x:v>1250 Avenue De La Station, Shawinigan, QC G9N 8K9; coordinate retained pending independent exact-address geocoding</x:v>
       </x:c>
     </x:row>
     <x:row r="217" ht="28">
@@ -27219,10 +28160,350 @@
         <x:v>Indianapolis, IN; GeoNames ID 4259418; exact plant coordinate should replace this point when verified</x:v>
       </x:c>
     </x:row>
+    <x:row r="389">
+      <x:c r="A389" t="n">
+        <x:v>389</x:v>
+      </x:c>
+      <x:c r="B389" t="str">
+        <x:v>Elysian - Capitol Hill Brewery</x:v>
+      </x:c>
+      <x:c r="C389" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D389" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E389" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F389" t="str">
+        <x:v>Seattle, WA; GeoNames ID 5809844; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="390">
+      <x:c r="A390" t="n">
+        <x:v>390</x:v>
+      </x:c>
+      <x:c r="B390" t="str">
+        <x:v>Wicked Weed - Original Brewpub Brewery</x:v>
+      </x:c>
+      <x:c r="C390" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D390" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E390" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F390" t="str">
+        <x:v>Asheville, NC; GeoNames ID 4453066; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="391">
+      <x:c r="A391" t="n">
+        <x:v>391</x:v>
+      </x:c>
+      <x:c r="B391" t="str">
+        <x:v>Wicked Weed - Funkatorium</x:v>
+      </x:c>
+      <x:c r="C391" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D391" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E391" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F391" t="str">
+        <x:v>Asheville, NC; GeoNames ID 4453066; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="392">
+      <x:c r="A392" t="n">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="B392" t="str">
+        <x:v>Wicked Weed West Production Brewery</x:v>
+      </x:c>
+      <x:c r="C392" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D392" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E392" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F392" t="str">
+        <x:v>Candler, NC; GeoNames ID 4459017; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="393">
+      <x:c r="A393" t="n">
+        <x:v>393</x:v>
+      </x:c>
+      <x:c r="B393" t="str">
+        <x:v>Karbach Brewery</x:v>
+      </x:c>
+      <x:c r="C393" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D393" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E393" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F393" t="str">
+        <x:v>Houston, TX; GeoNames ID 4699066; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="394">
+      <x:c r="A394" t="n">
+        <x:v>394</x:v>
+      </x:c>
+      <x:c r="B394" t="str">
+        <x:v>Devils Backbone - Basecamp Brewery</x:v>
+      </x:c>
+      <x:c r="C394" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D394" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E394" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F394" t="str">
+        <x:v>Roseland, VA; GeoNames ID 4782921; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="395">
+      <x:c r="A395" t="n">
+        <x:v>395</x:v>
+      </x:c>
+      <x:c r="B395" t="str">
+        <x:v>Devils Backbone - Outpost Production Brewery</x:v>
+      </x:c>
+      <x:c r="C395" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D395" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E395" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F395" t="str">
+        <x:v>Lexington, VA; GeoNames ID 4769339; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="396">
+      <x:c r="A396" t="n">
+        <x:v>396</x:v>
+      </x:c>
+      <x:c r="B396" t="str">
+        <x:v>Four Peaks - 8th Street Brewery</x:v>
+      </x:c>
+      <x:c r="C396" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D396" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E396" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F396" t="str">
+        <x:v>Tempe, AZ; GeoNames ID 5317058; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="397">
+      <x:c r="A397" t="n">
+        <x:v>397</x:v>
+      </x:c>
+      <x:c r="B397" t="str">
+        <x:v>Four Peaks - Wilson Production Brewery</x:v>
+      </x:c>
+      <x:c r="C397" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D397" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E397" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F397" t="str">
+        <x:v>Tempe, AZ; GeoNames ID 5317058; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="398">
+      <x:c r="A398" t="n">
+        <x:v>398</x:v>
+      </x:c>
+      <x:c r="B398" t="str">
+        <x:v>Cisco Brewers - Nantucket Brewery</x:v>
+      </x:c>
+      <x:c r="C398" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D398" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E398" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F398" t="str">
+        <x:v>Nantucket, MA; GeoNames ID 4944903; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="399">
+      <x:c r="A399" t="n">
+        <x:v>399</x:v>
+      </x:c>
+      <x:c r="B399" t="str">
+        <x:v>Casa La Rubia Brewery</x:v>
+      </x:c>
+      <x:c r="C399" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D399" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E399" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F399" t="str">
+        <x:v>Miami, FL; GeoNames ID 4164138; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="400">
+      <x:c r="A400" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="B400" t="str">
+        <x:v>Idaho Falls Barley Elevator</x:v>
+      </x:c>
+      <x:c r="C400" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D400" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E400" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F400" t="str">
+        <x:v>Idaho Falls, ID; GeoNames ID 5596475; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="401">
+      <x:c r="A401" t="n">
+        <x:v>401</x:v>
+      </x:c>
+      <x:c r="B401" t="str">
+        <x:v>Idaho Falls Malt Plant - Yellowstone Highway</x:v>
+      </x:c>
+      <x:c r="C401" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D401" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E401" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F401" t="str">
+        <x:v>Idaho Falls, ID; GeoNames ID 5596475; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="402">
+      <x:c r="A402" t="n">
+        <x:v>402</x:v>
+      </x:c>
+      <x:c r="B402" t="str">
+        <x:v>Idaho Falls Malt Plant - InteGrow</x:v>
+      </x:c>
+      <x:c r="C402" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D402" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E402" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F402" t="str">
+        <x:v>Idaho Falls, ID; GeoNames ID 5596475; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="403">
+      <x:c r="A403" t="n">
+        <x:v>403</x:v>
+      </x:c>
+      <x:c r="B403" t="str">
+        <x:v>Idaho Falls Seed Facility</x:v>
+      </x:c>
+      <x:c r="C403" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D403" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E403" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F403" t="str">
+        <x:v>Idaho Falls, ID; GeoNames ID 5596475; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="404">
+      <x:c r="A404" t="n">
+        <x:v>404</x:v>
+      </x:c>
+      <x:c r="B404" t="str">
+        <x:v>Elk Mountain Farms</x:v>
+      </x:c>
+      <x:c r="C404" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D404" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E404" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F404" t="str">
+        <x:v>Bonners Ferry, ID; GeoNames ID 5586496; exact facility coordinate should replace this point when verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="405">
+      <x:c r="A405" t="n">
+        <x:v>405</x:v>
+      </x:c>
+      <x:c r="B405" t="str">
+        <x:v>Jonesboro Rice Mill</x:v>
+      </x:c>
+      <x:c r="C405" t="str">
+        <x:v>Added</x:v>
+      </x:c>
+      <x:c r="D405" t="str">
+        <x:v>Arkansas DEQ postprocessed facility GPS</x:v>
+      </x:c>
+      <x:c r="E405" t="str">
+        <x:v>Exact facility / regulatory GPS</x:v>
+      </x:c>
+      <x:c r="F405" t="str">
+        <x:v>3723 County Road 905, Jonesboro, AR 72401; Arkansas DEQ NAD83 GPS</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R055b8fafc7594fe4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0901bf7b2be640c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Expand Crown North American facility network
</commit_message>
<xml_diff>
--- a/source-data/Strategic_End_User_Facilities_Bottler_Expansion_V3.xlsx
+++ b/source-data/Strategic_End_User_Facilities_Bottler_Expansion_V3.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Facilities v2" sheetId="1" r:id="Rd6dcfc7046dd4bb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Coverage" sheetId="2" r:id="R37f1391f71bf4cda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope &amp; Notes" sheetId="3" r:id="R0e1beeef49f746e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coordinate Audit" sheetId="4" r:id="Rd4228c53efa04fb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Facilities v2" sheetId="1" r:id="R9ea77d3233284a7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Coverage" sheetId="2" r:id="Ra100ac9905654834"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scope &amp; Notes" sheetId="3" r:id="Rf35cfde614b9413d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coordinate Audit" sheetId="4" r:id="Rdedd9a5d503a4c63"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -322,8 +322,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="StrategicFacilitiesV2" displayName="StrategicFacilitiesV2" ref="A1:P405" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:P405"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="StrategicFacilitiesV2" displayName="StrategicFacilitiesV2" ref="A1:P451" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:P451"/>
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="Vertical"/>
     <x:tableColumn id="2" name="Ultimate Parent"/>
@@ -347,8 +347,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="BottlerCoverage" displayName="BottlerCoverage" ref="A1:F15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F15"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="BottlerCoverage" displayName="BottlerCoverage" ref="A1:F16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F16"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Vertical"/>
     <x:tableColumn id="2" name="Ultimate Parent"/>
@@ -362,8 +362,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="CoordinateAuditTable" displayName="CoordinateAuditTable" ref="A1:F405" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F405"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="CoordinateAuditTable" displayName="CoordinateAuditTable" ref="A1:F451" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F451"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Excel Row"/>
     <x:tableColumn id="2" name="Facility Name"/>
@@ -3526,7 +3526,7 @@
         <x:v>Crown - Benton</x:v>
       </x:c>
       <x:c r="E64" s="2" t="str">
-        <x:v>Beverage Packaging</x:v>
+        <x:v>Transit Packaging</x:v>
       </x:c>
       <x:c r="F64" s="2"/>
       <x:c r="G64" s="2" t="str">
@@ -3549,12 +3549,14 @@
         <x:v>West</x:v>
       </x:c>
       <x:c r="N64" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O64" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P64" s="2"/>
+      <x:c r="P64" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="30" hidden="1">
       <x:c r="A65" s="2" t="str">
@@ -3593,12 +3595,14 @@
         <x:v>Midwest</x:v>
       </x:c>
       <x:c r="N65" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O65" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P65" s="2"/>
+      <x:c r="P65" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="30" hidden="1">
       <x:c r="A66" s="2" t="str">
@@ -3637,12 +3641,14 @@
         <x:v>Midwest</x:v>
       </x:c>
       <x:c r="N66" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O66" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P66" s="2"/>
+      <x:c r="P66" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="30" hidden="1">
       <x:c r="A67" s="2" t="str">
@@ -3681,12 +3687,14 @@
         <x:v>Midwest</x:v>
       </x:c>
       <x:c r="N67" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O67" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P67" s="2"/>
+      <x:c r="P67" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="30" hidden="1">
       <x:c r="A68" s="2" t="str">
@@ -3725,12 +3733,14 @@
         <x:v>Ohio Valley</x:v>
       </x:c>
       <x:c r="N68" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O68" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P68" s="2"/>
+      <x:c r="P68" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="30" hidden="1">
       <x:c r="A69" s="2" t="str">
@@ -3769,12 +3779,14 @@
         <x:v>Midwest</x:v>
       </x:c>
       <x:c r="N69" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O69" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P69" s="2"/>
+      <x:c r="P69" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="30" hidden="1">
       <x:c r="A70" s="2" t="str">
@@ -3813,12 +3825,14 @@
         <x:v>Midwest</x:v>
       </x:c>
       <x:c r="N70" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O70" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P70" s="2"/>
+      <x:c r="P70" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="30" hidden="1">
       <x:c r="A71" s="2" t="str">
@@ -3857,12 +3871,14 @@
         <x:v>Midwest</x:v>
       </x:c>
       <x:c r="N71" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O71" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P71" s="2"/>
+      <x:c r="P71" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="30" hidden="1">
       <x:c r="A72" s="2" t="str">
@@ -3901,12 +3917,14 @@
         <x:v>Northeast</x:v>
       </x:c>
       <x:c r="N72" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O72" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P72" s="2"/>
+      <x:c r="P72" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="30" hidden="1">
       <x:c r="A73" s="2" t="str">
@@ -3945,12 +3963,14 @@
         <x:v>Ohio Valley</x:v>
       </x:c>
       <x:c r="N73" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O73" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P73" s="2"/>
+      <x:c r="P73" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="30" hidden="1">
       <x:c r="A74" s="2" t="str">
@@ -3989,12 +4009,14 @@
         <x:v>Ohio Valley</x:v>
       </x:c>
       <x:c r="N74" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O74" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P74" s="2"/>
+      <x:c r="P74" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="30" hidden="1">
       <x:c r="A75" s="2" t="str">
@@ -4033,12 +4055,14 @@
         <x:v>Ohio Valley</x:v>
       </x:c>
       <x:c r="N75" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O75" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P75" s="2"/>
+      <x:c r="P75" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="76" ht="30" hidden="1">
       <x:c r="A76" s="2" t="str">
@@ -4077,12 +4101,14 @@
         <x:v>Ohio Valley</x:v>
       </x:c>
       <x:c r="N76" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O76" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P76" s="2"/>
+      <x:c r="P76" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="30" hidden="1">
       <x:c r="A77" s="2" t="str">
@@ -4121,12 +4147,14 @@
         <x:v>Northeast</x:v>
       </x:c>
       <x:c r="N77" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O77" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P77" s="2"/>
+      <x:c r="P77" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="78" ht="30" hidden="1">
       <x:c r="A78" s="2" t="str">
@@ -4165,12 +4193,14 @@
         <x:v>Northeast</x:v>
       </x:c>
       <x:c r="N78" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O78" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P78" s="2"/>
+      <x:c r="P78" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="79" ht="30" hidden="1">
       <x:c r="A79" s="2" t="str">
@@ -4209,12 +4239,14 @@
         <x:v>Southeast</x:v>
       </x:c>
       <x:c r="N79" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O79" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P79" s="2"/>
+      <x:c r="P79" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="80" ht="30" hidden="1">
       <x:c r="A80" s="2" t="str">
@@ -4244,21 +4276,23 @@
         <x:v>United States</x:v>
       </x:c>
       <x:c r="K80" s="15" t="n">
-        <x:v>34.05794</x:v>
+        <x:v>34.0576</x:v>
       </x:c>
       <x:c r="L80" s="15" t="n">
-        <x:v>-79.75312</x:v>
+        <x:v>-79.7534</x:v>
       </x:c>
       <x:c r="M80" s="2" t="str">
         <x:v>Southeast</x:v>
       </x:c>
       <x:c r="N80" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O80" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P80" s="2"/>
+      <x:c r="P80" s="2" t="str">
+        <x:v>Verified in Crown's current directory. Crown's page omits the minus sign on the Effingham longitude; the valid western-hemisphere longitude is retained and flagged here.</x:v>
+      </x:c>
     </x:row>
     <x:row r="81" ht="30" hidden="1">
       <x:c r="A81" s="2" t="str">
@@ -4297,12 +4331,14 @@
         <x:v>West</x:v>
       </x:c>
       <x:c r="N81" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O81" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P81" s="2"/>
+      <x:c r="P81" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="82" ht="30" hidden="1">
       <x:c r="A82" s="2" t="str">
@@ -4341,12 +4377,14 @@
         <x:v>West</x:v>
       </x:c>
       <x:c r="N82" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O82" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P82" s="2"/>
+      <x:c r="P82" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="83" ht="30" hidden="1">
       <x:c r="A83" s="2" t="str">
@@ -4385,12 +4423,14 @@
         <x:v>Northeast</x:v>
       </x:c>
       <x:c r="N83" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O83" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P83" s="2"/>
+      <x:c r="P83" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="84" ht="30" hidden="1">
       <x:c r="A84" s="2" t="str">
@@ -4429,12 +4469,14 @@
         <x:v>Northeast</x:v>
       </x:c>
       <x:c r="N84" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O84" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P84" s="2"/>
+      <x:c r="P84" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" ht="30" hidden="1">
       <x:c r="A85" s="2" t="str">
@@ -4473,12 +4515,14 @@
         <x:v>West</x:v>
       </x:c>
       <x:c r="N85" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O85" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P85" s="2"/>
+      <x:c r="P85" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="86" ht="30" hidden="1">
       <x:c r="A86" s="2" t="str">
@@ -4517,12 +4561,14 @@
         <x:v>Midwest</x:v>
       </x:c>
       <x:c r="N86" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O86" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P86" s="2"/>
+      <x:c r="P86" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="87" ht="30" hidden="1">
       <x:c r="A87" s="2" t="str">
@@ -4561,12 +4607,14 @@
         <x:v>West</x:v>
       </x:c>
       <x:c r="N87" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O87" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P87" s="2"/>
+      <x:c r="P87" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="88" ht="30" hidden="1">
       <x:c r="A88" s="2" t="str">
@@ -4582,7 +4630,7 @@
         <x:v>Crown - Calgary</x:v>
       </x:c>
       <x:c r="E88" s="2" t="str">
-        <x:v>Packaging</x:v>
+        <x:v>Beverage Packaging</x:v>
       </x:c>
       <x:c r="F88" s="2"/>
       <x:c r="G88" s="2" t="str">
@@ -4596,21 +4644,23 @@
         <x:v>Canada</x:v>
       </x:c>
       <x:c r="K88" s="15" t="n">
-        <x:v>51.05011</x:v>
+        <x:v>51.0447331</x:v>
       </x:c>
       <x:c r="L88" s="15" t="n">
-        <x:v>-114.08529</x:v>
+        <x:v>-114.0718831</x:v>
       </x:c>
       <x:c r="M88" s="2" t="str">
         <x:v>Canada</x:v>
       </x:c>
       <x:c r="N88" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O88" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P88" s="2"/>
+      <x:c r="P88" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="89" ht="30" hidden="1">
       <x:c r="A89" s="2" t="str">
@@ -4626,7 +4676,7 @@
         <x:v>Crown - Halton Hills</x:v>
       </x:c>
       <x:c r="E89" s="2" t="str">
-        <x:v>Packaging</x:v>
+        <x:v>Transit Packaging</x:v>
       </x:c>
       <x:c r="F89" s="2"/>
       <x:c r="G89" s="2" t="str">
@@ -4640,21 +4690,23 @@
         <x:v>Canada</x:v>
       </x:c>
       <x:c r="K89" s="15" t="n">
-        <x:v>43.6403</x:v>
+        <x:v>43.6503</x:v>
       </x:c>
       <x:c r="L89" s="15" t="n">
-        <x:v>-79.93146</x:v>
+        <x:v>-79.9036</x:v>
       </x:c>
       <x:c r="M89" s="2" t="str">
         <x:v>Canada</x:v>
       </x:c>
       <x:c r="N89" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O89" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P89" s="2"/>
+      <x:c r="P89" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="90" ht="30" hidden="1">
       <x:c r="A90" s="2" t="str">
@@ -4670,7 +4722,7 @@
         <x:v>Crown - Toronto</x:v>
       </x:c>
       <x:c r="E90" s="2" t="str">
-        <x:v>Packaging / office</x:v>
+        <x:v>Beverage Packaging</x:v>
       </x:c>
       <x:c r="F90" s="2"/>
       <x:c r="G90" s="2" t="str">
@@ -4684,21 +4736,23 @@
         <x:v>Canada</x:v>
       </x:c>
       <x:c r="K90" s="15" t="n">
-        <x:v>43.70643</x:v>
+        <x:v>43.653226</x:v>
       </x:c>
       <x:c r="L90" s="15" t="n">
-        <x:v>-79.39864</x:v>
+        <x:v>-79.3831843</x:v>
       </x:c>
       <x:c r="M90" s="2" t="str">
         <x:v>Canada</x:v>
       </x:c>
       <x:c r="N90" s="2" t="str">
-        <x:v>Verified official location - street address pending</x:v>
+        <x:v>Verified - official Crown directory</x:v>
       </x:c>
       <x:c r="O90" s="2" t="str">
         <x:v>https://www.crowncork.com/about/global-locations</x:v>
       </x:c>
-      <x:c r="P90" s="2"/>
+      <x:c r="P90" s="2" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
     </x:row>
     <x:row r="91" ht="15" hidden="1">
       <x:c r="A91" s="2" t="str">
@@ -19960,6 +20014,2122 @@
       </x:c>
       <x:c r="P405" t="str">
         <x:v>Current A-B brewing page confirms the Jonesboro rice mill; Arkansas DEQ provides the street address and postprocessed facility GPS coordinate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="406">
+      <x:c r="A406" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B406" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C406" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D406" t="str">
+        <x:v>Crown - Fordyce</x:v>
+      </x:c>
+      <x:c r="E406" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F406"/>
+      <x:c r="G406" t="str">
+        <x:v>Fordyce</x:v>
+      </x:c>
+      <x:c r="H406" t="str">
+        <x:v>AR</x:v>
+      </x:c>
+      <x:c r="I406"/>
+      <x:c r="J406" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K406" t="n">
+        <x:v>33.8137295</x:v>
+      </x:c>
+      <x:c r="L406" t="n">
+        <x:v>-92.4129746</x:v>
+      </x:c>
+      <x:c r="M406" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="N406" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O406" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P406" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="407">
+      <x:c r="A407" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B407" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C407" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D407" t="str">
+        <x:v>Crown - Sheridan</x:v>
+      </x:c>
+      <x:c r="E407" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F407"/>
+      <x:c r="G407" t="str">
+        <x:v>Sheridan</x:v>
+      </x:c>
+      <x:c r="H407" t="str">
+        <x:v>AR</x:v>
+      </x:c>
+      <x:c r="I407"/>
+      <x:c r="J407" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K407" t="n">
+        <x:v>34.3068334</x:v>
+      </x:c>
+      <x:c r="L407" t="n">
+        <x:v>-92.3991409</x:v>
+      </x:c>
+      <x:c r="M407" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="N407" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O407" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P407" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="408">
+      <x:c r="A408" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B408" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C408" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D408" t="str">
+        <x:v>Crown - Phoenix</x:v>
+      </x:c>
+      <x:c r="E408" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F408"/>
+      <x:c r="G408" t="str">
+        <x:v>Phoenix</x:v>
+      </x:c>
+      <x:c r="H408" t="str">
+        <x:v>AZ</x:v>
+      </x:c>
+      <x:c r="I408"/>
+      <x:c r="J408" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K408" t="n">
+        <x:v>33.4483771</x:v>
+      </x:c>
+      <x:c r="L408" t="n">
+        <x:v>-112.0740373</x:v>
+      </x:c>
+      <x:c r="M408" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N408" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O408" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P408" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="409">
+      <x:c r="A409" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B409" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C409" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D409" t="str">
+        <x:v>Crown - Bay Point</x:v>
+      </x:c>
+      <x:c r="E409" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F409"/>
+      <x:c r="G409" t="str">
+        <x:v>Bay Point</x:v>
+      </x:c>
+      <x:c r="H409" t="str">
+        <x:v>CA</x:v>
+      </x:c>
+      <x:c r="I409"/>
+      <x:c r="J409" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K409" t="n">
+        <x:v>38.0290872</x:v>
+      </x:c>
+      <x:c r="L409" t="n">
+        <x:v>-121.9616274</x:v>
+      </x:c>
+      <x:c r="M409" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N409" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O409" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P409" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="410">
+      <x:c r="A410" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B410" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C410" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D410" t="str">
+        <x:v>Crown - Stockton</x:v>
+      </x:c>
+      <x:c r="E410" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F410"/>
+      <x:c r="G410" t="str">
+        <x:v>Stockton</x:v>
+      </x:c>
+      <x:c r="H410" t="str">
+        <x:v>CA</x:v>
+      </x:c>
+      <x:c r="I410"/>
+      <x:c r="J410" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K410" t="n">
+        <x:v>37.9577016</x:v>
+      </x:c>
+      <x:c r="L410" t="n">
+        <x:v>-121.2907796</x:v>
+      </x:c>
+      <x:c r="M410" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N410" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O410" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P410" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="411">
+      <x:c r="A411" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B411" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C411" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D411" t="str">
+        <x:v>Crown - Douglasville</x:v>
+      </x:c>
+      <x:c r="E411" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F411"/>
+      <x:c r="G411" t="str">
+        <x:v>Douglasville</x:v>
+      </x:c>
+      <x:c r="H411" t="str">
+        <x:v>GA</x:v>
+      </x:c>
+      <x:c r="I411"/>
+      <x:c r="J411" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K411" t="n">
+        <x:v>33.7514966</x:v>
+      </x:c>
+      <x:c r="L411" t="n">
+        <x:v>-84.7477136</x:v>
+      </x:c>
+      <x:c r="M411" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N411" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O411" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P411" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="412">
+      <x:c r="A412" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B412" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C412" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D412" t="str">
+        <x:v>Crown - LaGrange</x:v>
+      </x:c>
+      <x:c r="E412" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F412"/>
+      <x:c r="G412" t="str">
+        <x:v>LaGrange</x:v>
+      </x:c>
+      <x:c r="H412" t="str">
+        <x:v>GA</x:v>
+      </x:c>
+      <x:c r="I412"/>
+      <x:c r="J412" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K412" t="n">
+        <x:v>33.0362218</x:v>
+      </x:c>
+      <x:c r="L412" t="n">
+        <x:v>-85.0322444</x:v>
+      </x:c>
+      <x:c r="M412" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N412" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O412" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P412" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="413">
+      <x:c r="A413" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B413" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C413" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D413" t="str">
+        <x:v>Crown - Macon</x:v>
+      </x:c>
+      <x:c r="E413" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F413"/>
+      <x:c r="G413" t="str">
+        <x:v>Macon</x:v>
+      </x:c>
+      <x:c r="H413" t="str">
+        <x:v>GA</x:v>
+      </x:c>
+      <x:c r="I413"/>
+      <x:c r="J413" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K413" t="n">
+        <x:v>32.8406946</x:v>
+      </x:c>
+      <x:c r="L413" t="n">
+        <x:v>-83.6324022</x:v>
+      </x:c>
+      <x:c r="M413" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N413" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O413" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P413" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="414">
+      <x:c r="A414" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B414" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C414" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D414" t="str">
+        <x:v>Crown - Bridgeview</x:v>
+      </x:c>
+      <x:c r="E414" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F414"/>
+      <x:c r="G414" t="str">
+        <x:v>Bridgeview</x:v>
+      </x:c>
+      <x:c r="H414" t="str">
+        <x:v>IL</x:v>
+      </x:c>
+      <x:c r="I414"/>
+      <x:c r="J414" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K414" t="n">
+        <x:v>41.7500323</x:v>
+      </x:c>
+      <x:c r="L414" t="n">
+        <x:v>-87.8042216</x:v>
+      </x:c>
+      <x:c r="M414" t="str">
+        <x:v>Midwest</x:v>
+      </x:c>
+      <x:c r="N414" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O414" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P414" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="415">
+      <x:c r="A415" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B415" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C415" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D415" t="str">
+        <x:v>Crown - Dixmoor</x:v>
+      </x:c>
+      <x:c r="E415" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F415"/>
+      <x:c r="G415" t="str">
+        <x:v>Dixmoor</x:v>
+      </x:c>
+      <x:c r="H415" t="str">
+        <x:v>IL</x:v>
+      </x:c>
+      <x:c r="I415"/>
+      <x:c r="J415" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K415" t="n">
+        <x:v>41.6298973</x:v>
+      </x:c>
+      <x:c r="L415" t="n">
+        <x:v>-87.6609098</x:v>
+      </x:c>
+      <x:c r="M415" t="str">
+        <x:v>Midwest</x:v>
+      </x:c>
+      <x:c r="N415" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O415" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P415" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="416">
+      <x:c r="A416" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B416" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C416" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D416" t="str">
+        <x:v>Crown - Roselle</x:v>
+      </x:c>
+      <x:c r="E416" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F416"/>
+      <x:c r="G416" t="str">
+        <x:v>Roselle</x:v>
+      </x:c>
+      <x:c r="H416" t="str">
+        <x:v>IL</x:v>
+      </x:c>
+      <x:c r="I416"/>
+      <x:c r="J416" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K416" t="n">
+        <x:v>41.9847504</x:v>
+      </x:c>
+      <x:c r="L416" t="n">
+        <x:v>-88.0797933</x:v>
+      </x:c>
+      <x:c r="M416" t="str">
+        <x:v>Midwest</x:v>
+      </x:c>
+      <x:c r="N416" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O416" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P416" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="417">
+      <x:c r="A417" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B417" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C417" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D417" t="str">
+        <x:v>Crown - Elkhart</x:v>
+      </x:c>
+      <x:c r="E417" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F417"/>
+      <x:c r="G417" t="str">
+        <x:v>Elkhart</x:v>
+      </x:c>
+      <x:c r="H417" t="str">
+        <x:v>IN</x:v>
+      </x:c>
+      <x:c r="I417"/>
+      <x:c r="J417" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K417" t="n">
+        <x:v>41.6873832</x:v>
+      </x:c>
+      <x:c r="L417" t="n">
+        <x:v>-85.973517</x:v>
+      </x:c>
+      <x:c r="M417" t="str">
+        <x:v>Midwest</x:v>
+      </x:c>
+      <x:c r="N417" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O417" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P417" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="418">
+      <x:c r="A418" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B418" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C418" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D418" t="str">
+        <x:v>Crown - Gary</x:v>
+      </x:c>
+      <x:c r="E418" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F418"/>
+      <x:c r="G418" t="str">
+        <x:v>Gary</x:v>
+      </x:c>
+      <x:c r="H418" t="str">
+        <x:v>IN</x:v>
+      </x:c>
+      <x:c r="I418"/>
+      <x:c r="J418" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K418" t="n">
+        <x:v>41.6020403</x:v>
+      </x:c>
+      <x:c r="L418" t="n">
+        <x:v>-87.3371523</x:v>
+      </x:c>
+      <x:c r="M418" t="str">
+        <x:v>Midwest</x:v>
+      </x:c>
+      <x:c r="N418" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O418" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P418" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="419">
+      <x:c r="A419" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B419" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C419" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D419" t="str">
+        <x:v>Crown - Florence</x:v>
+      </x:c>
+      <x:c r="E419" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F419"/>
+      <x:c r="G419" t="str">
+        <x:v>Florence</x:v>
+      </x:c>
+      <x:c r="H419" t="str">
+        <x:v>KY</x:v>
+      </x:c>
+      <x:c r="I419"/>
+      <x:c r="J419" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K419" t="n">
+        <x:v>38.9989499</x:v>
+      </x:c>
+      <x:c r="L419" t="n">
+        <x:v>-84.6266111</x:v>
+      </x:c>
+      <x:c r="M419" t="str">
+        <x:v>Ohio Valley</x:v>
+      </x:c>
+      <x:c r="N419" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O419" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P419" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="420">
+      <x:c r="A420" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B420" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C420" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D420" t="str">
+        <x:v>Crown - Monroe</x:v>
+      </x:c>
+      <x:c r="E420" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F420"/>
+      <x:c r="G420" t="str">
+        <x:v>Monroe</x:v>
+      </x:c>
+      <x:c r="H420" t="str">
+        <x:v>LA</x:v>
+      </x:c>
+      <x:c r="I420"/>
+      <x:c r="J420" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K420" t="n">
+        <x:v>32.5093109</x:v>
+      </x:c>
+      <x:c r="L420" t="n">
+        <x:v>-92.1193012</x:v>
+      </x:c>
+      <x:c r="M420" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="N420" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O420" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P420" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="421">
+      <x:c r="A421" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B421" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C421" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D421" t="str">
+        <x:v>Crown - Belcamp</x:v>
+      </x:c>
+      <x:c r="E421" t="str">
+        <x:v>Promotional Tins</x:v>
+      </x:c>
+      <x:c r="F421"/>
+      <x:c r="G421" t="str">
+        <x:v>Belcamp</x:v>
+      </x:c>
+      <x:c r="H421" t="str">
+        <x:v>MD</x:v>
+      </x:c>
+      <x:c r="I421"/>
+      <x:c r="J421" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K421" t="n">
+        <x:v>39.4737199</x:v>
+      </x:c>
+      <x:c r="L421" t="n">
+        <x:v>-76.2413446</x:v>
+      </x:c>
+      <x:c r="M421" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="N421" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O421" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P421" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="422">
+      <x:c r="A422" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B422" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C422" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D422" t="str">
+        <x:v>Crown - Brighton</x:v>
+      </x:c>
+      <x:c r="E422" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F422"/>
+      <x:c r="G422" t="str">
+        <x:v>Brighton</x:v>
+      </x:c>
+      <x:c r="H422" t="str">
+        <x:v>MI</x:v>
+      </x:c>
+      <x:c r="I422"/>
+      <x:c r="J422" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K422" t="n">
+        <x:v>42.5294773</x:v>
+      </x:c>
+      <x:c r="L422" t="n">
+        <x:v>-83.7802214</x:v>
+      </x:c>
+      <x:c r="M422" t="str">
+        <x:v>Midwest</x:v>
+      </x:c>
+      <x:c r="N422" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O422" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P422" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="423">
+      <x:c r="A423" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B423" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C423" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D423" t="str">
+        <x:v>Crown - Eden</x:v>
+      </x:c>
+      <x:c r="E423" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F423"/>
+      <x:c r="G423" t="str">
+        <x:v>Eden</x:v>
+      </x:c>
+      <x:c r="H423" t="str">
+        <x:v>NC</x:v>
+      </x:c>
+      <x:c r="I423"/>
+      <x:c r="J423" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K423" t="n">
+        <x:v>36.4884715</x:v>
+      </x:c>
+      <x:c r="L423" t="n">
+        <x:v>-79.7667026</x:v>
+      </x:c>
+      <x:c r="M423" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N423" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O423" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P423" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="424">
+      <x:c r="A424" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B424" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C424" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D424" t="str">
+        <x:v>Crown - Salisbury</x:v>
+      </x:c>
+      <x:c r="E424" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F424"/>
+      <x:c r="G424" t="str">
+        <x:v>Salisbury</x:v>
+      </x:c>
+      <x:c r="H424" t="str">
+        <x:v>NC</x:v>
+      </x:c>
+      <x:c r="I424"/>
+      <x:c r="J424" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K424" t="n">
+        <x:v>35.6709727</x:v>
+      </x:c>
+      <x:c r="L424" t="n">
+        <x:v>-80.4742261</x:v>
+      </x:c>
+      <x:c r="M424" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N424" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O424" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P424" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="425">
+      <x:c r="A425" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B425" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C425" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D425" t="str">
+        <x:v>Crown - Irvington</x:v>
+      </x:c>
+      <x:c r="E425" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F425"/>
+      <x:c r="G425" t="str">
+        <x:v>Irvington</x:v>
+      </x:c>
+      <x:c r="H425" t="str">
+        <x:v>NJ</x:v>
+      </x:c>
+      <x:c r="I425"/>
+      <x:c r="J425" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K425" t="n">
+        <x:v>40.7263249</x:v>
+      </x:c>
+      <x:c r="L425" t="n">
+        <x:v>-74.2286435</x:v>
+      </x:c>
+      <x:c r="M425" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="N425" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O425" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P425" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="426">
+      <x:c r="A426" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B426" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C426" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D426" t="str">
+        <x:v>Crown - Mesquite</x:v>
+      </x:c>
+      <x:c r="E426" t="str">
+        <x:v>Beverage Packaging</x:v>
+      </x:c>
+      <x:c r="F426"/>
+      <x:c r="G426" t="str">
+        <x:v>Mesquite</x:v>
+      </x:c>
+      <x:c r="H426" t="str">
+        <x:v>NV</x:v>
+      </x:c>
+      <x:c r="I426"/>
+      <x:c r="J426" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K426" t="n">
+        <x:v>36.8824</x:v>
+      </x:c>
+      <x:c r="L426" t="n">
+        <x:v>-114.1202</x:v>
+      </x:c>
+      <x:c r="M426" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N426" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O426" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P426" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="427">
+      <x:c r="A427" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B427" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C427" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D427" t="str">
+        <x:v>Crown - Cleveland</x:v>
+      </x:c>
+      <x:c r="E427" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F427"/>
+      <x:c r="G427" t="str">
+        <x:v>Cleveland</x:v>
+      </x:c>
+      <x:c r="H427" t="str">
+        <x:v>OH</x:v>
+      </x:c>
+      <x:c r="I427"/>
+      <x:c r="J427" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K427" t="n">
+        <x:v>41.49932</x:v>
+      </x:c>
+      <x:c r="L427" t="n">
+        <x:v>-81.6943605</x:v>
+      </x:c>
+      <x:c r="M427" t="str">
+        <x:v>Ohio Valley</x:v>
+      </x:c>
+      <x:c r="N427" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O427" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P427" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="428">
+      <x:c r="A428" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B428" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C428" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D428" t="str">
+        <x:v>Crown - Loveland</x:v>
+      </x:c>
+      <x:c r="E428" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F428"/>
+      <x:c r="G428" t="str">
+        <x:v>Loveland</x:v>
+      </x:c>
+      <x:c r="H428" t="str">
+        <x:v>OH</x:v>
+      </x:c>
+      <x:c r="I428"/>
+      <x:c r="J428" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K428" t="n">
+        <x:v>39.2689476</x:v>
+      </x:c>
+      <x:c r="L428" t="n">
+        <x:v>-84.263826</x:v>
+      </x:c>
+      <x:c r="M428" t="str">
+        <x:v>Ohio Valley</x:v>
+      </x:c>
+      <x:c r="N428" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O428" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P428" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="429">
+      <x:c r="A429" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B429" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C429" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D429" t="str">
+        <x:v>Crown - West Chester</x:v>
+      </x:c>
+      <x:c r="E429" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F429"/>
+      <x:c r="G429" t="str">
+        <x:v>West Chester</x:v>
+      </x:c>
+      <x:c r="H429" t="str">
+        <x:v>OH</x:v>
+      </x:c>
+      <x:c r="I429"/>
+      <x:c r="J429" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K429" t="n">
+        <x:v>39.3321262</x:v>
+      </x:c>
+      <x:c r="L429" t="n">
+        <x:v>-84.4172666</x:v>
+      </x:c>
+      <x:c r="M429" t="str">
+        <x:v>Ohio Valley</x:v>
+      </x:c>
+      <x:c r="N429" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O429" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P429" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="430">
+      <x:c r="A430" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B430" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C430" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D430" t="str">
+        <x:v>Crown - Hazleton</x:v>
+      </x:c>
+      <x:c r="E430" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F430"/>
+      <x:c r="G430" t="str">
+        <x:v>Hazleton</x:v>
+      </x:c>
+      <x:c r="H430" t="str">
+        <x:v>PA</x:v>
+      </x:c>
+      <x:c r="I430"/>
+      <x:c r="J430" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K430" t="n">
+        <x:v>40.9584181</x:v>
+      </x:c>
+      <x:c r="L430" t="n">
+        <x:v>-75.9746472</x:v>
+      </x:c>
+      <x:c r="M430" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="N430" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O430" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P430" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="431">
+      <x:c r="A431" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B431" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C431" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D431" t="str">
+        <x:v>Crown - South Canaan</x:v>
+      </x:c>
+      <x:c r="E431" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F431"/>
+      <x:c r="G431" t="str">
+        <x:v>South Canaan</x:v>
+      </x:c>
+      <x:c r="H431" t="str">
+        <x:v>PA</x:v>
+      </x:c>
+      <x:c r="I431"/>
+      <x:c r="J431" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K431" t="n">
+        <x:v>41.5191717</x:v>
+      </x:c>
+      <x:c r="L431" t="n">
+        <x:v>-75.4111644</x:v>
+      </x:c>
+      <x:c r="M431" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="N431" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O431" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P431" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="432">
+      <x:c r="A432" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B432" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C432" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D432" t="str">
+        <x:v>Crown - East Providence</x:v>
+      </x:c>
+      <x:c r="E432" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F432"/>
+      <x:c r="G432" t="str">
+        <x:v>East Providence</x:v>
+      </x:c>
+      <x:c r="H432" t="str">
+        <x:v>RI</x:v>
+      </x:c>
+      <x:c r="I432"/>
+      <x:c r="J432" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K432" t="n">
+        <x:v>41.8137116</x:v>
+      </x:c>
+      <x:c r="L432" t="n">
+        <x:v>-71.3700545</x:v>
+      </x:c>
+      <x:c r="M432" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="N432" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O432" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P432" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="433">
+      <x:c r="A433" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B433" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C433" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D433" t="str">
+        <x:v>Crown - Darlington</x:v>
+      </x:c>
+      <x:c r="E433" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F433"/>
+      <x:c r="G433" t="str">
+        <x:v>Darlington</x:v>
+      </x:c>
+      <x:c r="H433" t="str">
+        <x:v>SC</x:v>
+      </x:c>
+      <x:c r="I433"/>
+      <x:c r="J433" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K433" t="n">
+        <x:v>34.3003526</x:v>
+      </x:c>
+      <x:c r="L433" t="n">
+        <x:v>-79.8757116</x:v>
+      </x:c>
+      <x:c r="M433" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N433" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O433" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P433" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="434">
+      <x:c r="A434" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B434" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C434" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D434" t="str">
+        <x:v>Crown - Greer</x:v>
+      </x:c>
+      <x:c r="E434" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F434"/>
+      <x:c r="G434" t="str">
+        <x:v>Greer</x:v>
+      </x:c>
+      <x:c r="H434" t="str">
+        <x:v>SC</x:v>
+      </x:c>
+      <x:c r="I434"/>
+      <x:c r="J434" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K434" t="n">
+        <x:v>34.9387279</x:v>
+      </x:c>
+      <x:c r="L434" t="n">
+        <x:v>-82.2270568</x:v>
+      </x:c>
+      <x:c r="M434" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N434" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O434" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P434" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="435">
+      <x:c r="A435" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B435" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C435" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D435" t="str">
+        <x:v>Crown - Latta</x:v>
+      </x:c>
+      <x:c r="E435" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F435"/>
+      <x:c r="G435" t="str">
+        <x:v>Latta</x:v>
+      </x:c>
+      <x:c r="H435" t="str">
+        <x:v>SC</x:v>
+      </x:c>
+      <x:c r="I435"/>
+      <x:c r="J435" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K435" t="n">
+        <x:v>34.3371047</x:v>
+      </x:c>
+      <x:c r="L435" t="n">
+        <x:v>-79.4311616</x:v>
+      </x:c>
+      <x:c r="M435" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N435" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O435" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P435" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="436">
+      <x:c r="A436" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B436" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C436" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D436" t="str">
+        <x:v>Crown - Spartanburg</x:v>
+      </x:c>
+      <x:c r="E436" t="str">
+        <x:v>Aerosol Cans</x:v>
+      </x:c>
+      <x:c r="F436"/>
+      <x:c r="G436" t="str">
+        <x:v>Spartanburg</x:v>
+      </x:c>
+      <x:c r="H436" t="str">
+        <x:v>SC</x:v>
+      </x:c>
+      <x:c r="I436"/>
+      <x:c r="J436" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K436" t="n">
+        <x:v>34.9495672</x:v>
+      </x:c>
+      <x:c r="L436" t="n">
+        <x:v>-81.9320482</x:v>
+      </x:c>
+      <x:c r="M436" t="str">
+        <x:v>Southeast</x:v>
+      </x:c>
+      <x:c r="N436" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O436" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P436" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="437">
+      <x:c r="A437" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B437" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C437" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D437" t="str">
+        <x:v>Crown - Orange</x:v>
+      </x:c>
+      <x:c r="E437" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F437"/>
+      <x:c r="G437" t="str">
+        <x:v>Orange</x:v>
+      </x:c>
+      <x:c r="H437" t="str">
+        <x:v>TX</x:v>
+      </x:c>
+      <x:c r="I437"/>
+      <x:c r="J437" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K437" t="n">
+        <x:v>30.0929879</x:v>
+      </x:c>
+      <x:c r="L437" t="n">
+        <x:v>-93.7365549</x:v>
+      </x:c>
+      <x:c r="M437" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="N437" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O437" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P437" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="438">
+      <x:c r="A438" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B438" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C438" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D438" t="str">
+        <x:v>Crown - San Antonio</x:v>
+      </x:c>
+      <x:c r="E438" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F438"/>
+      <x:c r="G438" t="str">
+        <x:v>San Antonio</x:v>
+      </x:c>
+      <x:c r="H438" t="str">
+        <x:v>TX</x:v>
+      </x:c>
+      <x:c r="I438"/>
+      <x:c r="J438" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K438" t="n">
+        <x:v>29.4251905</x:v>
+      </x:c>
+      <x:c r="L438" t="n">
+        <x:v>-98.4945922</x:v>
+      </x:c>
+      <x:c r="M438" t="str">
+        <x:v>South</x:v>
+      </x:c>
+      <x:c r="N438" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O438" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P438" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="439">
+      <x:c r="A439" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B439" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C439" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D439" t="str">
+        <x:v>Crown - Forest</x:v>
+      </x:c>
+      <x:c r="E439" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F439"/>
+      <x:c r="G439" t="str">
+        <x:v>Forest</x:v>
+      </x:c>
+      <x:c r="H439" t="str">
+        <x:v>VA</x:v>
+      </x:c>
+      <x:c r="I439"/>
+      <x:c r="J439" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K439" t="n">
+        <x:v>37.3638</x:v>
+      </x:c>
+      <x:c r="L439" t="n">
+        <x:v>-79.2897</x:v>
+      </x:c>
+      <x:c r="M439" t="str">
+        <x:v>Northeast</x:v>
+      </x:c>
+      <x:c r="N439" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O439" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P439" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="440">
+      <x:c r="A440" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B440" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C440" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D440" t="str">
+        <x:v>Crown - Danville</x:v>
+      </x:c>
+      <x:c r="E440" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F440"/>
+      <x:c r="G440" t="str">
+        <x:v>Danville</x:v>
+      </x:c>
+      <x:c r="H440" t="str">
+        <x:v>WA</x:v>
+      </x:c>
+      <x:c r="I440"/>
+      <x:c r="J440" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K440" t="n">
+        <x:v>48.9921647</x:v>
+      </x:c>
+      <x:c r="L440" t="n">
+        <x:v>-118.5081439</x:v>
+      </x:c>
+      <x:c r="M440" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N440" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O440" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P440" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="441">
+      <x:c r="A441" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B441" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C441" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D441" t="str">
+        <x:v>Crown - Woodland</x:v>
+      </x:c>
+      <x:c r="E441" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F441"/>
+      <x:c r="G441" t="str">
+        <x:v>Woodland</x:v>
+      </x:c>
+      <x:c r="H441" t="str">
+        <x:v>WA</x:v>
+      </x:c>
+      <x:c r="I441"/>
+      <x:c r="J441" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K441" t="n">
+        <x:v>45.9045591</x:v>
+      </x:c>
+      <x:c r="L441" t="n">
+        <x:v>-122.7439912</x:v>
+      </x:c>
+      <x:c r="M441" t="str">
+        <x:v>West</x:v>
+      </x:c>
+      <x:c r="N441" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O441" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P441" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="442">
+      <x:c r="A442" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B442" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C442" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D442" t="str">
+        <x:v>Crown - Oshkosh</x:v>
+      </x:c>
+      <x:c r="E442" t="str">
+        <x:v>Food Cans</x:v>
+      </x:c>
+      <x:c r="F442"/>
+      <x:c r="G442" t="str">
+        <x:v>Oshkosh</x:v>
+      </x:c>
+      <x:c r="H442" t="str">
+        <x:v>WI</x:v>
+      </x:c>
+      <x:c r="I442"/>
+      <x:c r="J442" t="str">
+        <x:v>United States</x:v>
+      </x:c>
+      <x:c r="K442" t="n">
+        <x:v>44.0247062</x:v>
+      </x:c>
+      <x:c r="L442" t="n">
+        <x:v>-88.5426136</x:v>
+      </x:c>
+      <x:c r="M442" t="str">
+        <x:v>Midwest</x:v>
+      </x:c>
+      <x:c r="N442" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O442" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P442" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="443">
+      <x:c r="A443" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B443" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C443" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D443" t="str">
+        <x:v>Crown - Ensenada</x:v>
+      </x:c>
+      <x:c r="E443" t="str">
+        <x:v>Beverage Packaging</x:v>
+      </x:c>
+      <x:c r="F443"/>
+      <x:c r="G443" t="str">
+        <x:v>Ensenada</x:v>
+      </x:c>
+      <x:c r="H443" t="str">
+        <x:v>BCN</x:v>
+      </x:c>
+      <x:c r="I443"/>
+      <x:c r="J443" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="K443" t="n">
+        <x:v>31.8667427</x:v>
+      </x:c>
+      <x:c r="L443" t="n">
+        <x:v>-116.5963713</x:v>
+      </x:c>
+      <x:c r="M443" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="N443" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O443" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P443" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="444">
+      <x:c r="A444" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B444" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C444" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D444" t="str">
+        <x:v>Crown - Chihuahua</x:v>
+      </x:c>
+      <x:c r="E444" t="str">
+        <x:v>Beverage Packaging</x:v>
+      </x:c>
+      <x:c r="F444"/>
+      <x:c r="G444" t="str">
+        <x:v>Chihuahua</x:v>
+      </x:c>
+      <x:c r="H444" t="str">
+        <x:v>CHH</x:v>
+      </x:c>
+      <x:c r="I444"/>
+      <x:c r="J444" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="K444" t="n">
+        <x:v>28.6352778</x:v>
+      </x:c>
+      <x:c r="L444" t="n">
+        <x:v>-106.0888889</x:v>
+      </x:c>
+      <x:c r="M444" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="N444" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O444" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P444" t="str">
+        <x:v>Verified in Crown's current directory. Crown's published Chihuahua longitude is outside Chihuahua; GeoNames city coordinate used rather than reproducing the directory error.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="445">
+      <x:c r="A445" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B445" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C445" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D445" t="str">
+        <x:v>Crown - Guadalajara</x:v>
+      </x:c>
+      <x:c r="E445" t="str">
+        <x:v>Beverage Packaging</x:v>
+      </x:c>
+      <x:c r="F445"/>
+      <x:c r="G445" t="str">
+        <x:v>Guadalajara</x:v>
+      </x:c>
+      <x:c r="H445" t="str">
+        <x:v>JAL</x:v>
+      </x:c>
+      <x:c r="I445"/>
+      <x:c r="J445" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="K445" t="n">
+        <x:v>20.6596988</x:v>
+      </x:c>
+      <x:c r="L445" t="n">
+        <x:v>-103.3496092</x:v>
+      </x:c>
+      <x:c r="M445" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="N445" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O445" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P445" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="446">
+      <x:c r="A446" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B446" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C446" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D446" t="str">
+        <x:v>Crown - Toluca</x:v>
+      </x:c>
+      <x:c r="E446" t="str">
+        <x:v>Beverage Packaging / Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F446"/>
+      <x:c r="G446" t="str">
+        <x:v>Toluca</x:v>
+      </x:c>
+      <x:c r="H446" t="str">
+        <x:v>MEX</x:v>
+      </x:c>
+      <x:c r="I446"/>
+      <x:c r="J446" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="K446" t="n">
+        <x:v>19.2826098</x:v>
+      </x:c>
+      <x:c r="L446" t="n">
+        <x:v>-99.6556653</x:v>
+      </x:c>
+      <x:c r="M446" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="N446" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O446" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P446" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="447">
+      <x:c r="A447" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B447" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C447" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D447" t="str">
+        <x:v>Crown - Ciénega de Flores</x:v>
+      </x:c>
+      <x:c r="E447" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F447"/>
+      <x:c r="G447" t="str">
+        <x:v>Ciénega de Flores</x:v>
+      </x:c>
+      <x:c r="H447" t="str">
+        <x:v>NLE</x:v>
+      </x:c>
+      <x:c r="I447"/>
+      <x:c r="J447" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="K447" t="n">
+        <x:v>25.9543957</x:v>
+      </x:c>
+      <x:c r="L447" t="n">
+        <x:v>-100.166333</x:v>
+      </x:c>
+      <x:c r="M447" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="N447" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O447" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P447" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="448">
+      <x:c r="A448" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B448" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C448" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D448" t="str">
+        <x:v>Crown - Monterrey</x:v>
+      </x:c>
+      <x:c r="E448" t="str">
+        <x:v>Beverage Packaging / Closures &amp; Capping</x:v>
+      </x:c>
+      <x:c r="F448"/>
+      <x:c r="G448" t="str">
+        <x:v>Monterrey</x:v>
+      </x:c>
+      <x:c r="H448" t="str">
+        <x:v>NLE</x:v>
+      </x:c>
+      <x:c r="I448"/>
+      <x:c r="J448" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="K448" t="n">
+        <x:v>25.6866142</x:v>
+      </x:c>
+      <x:c r="L448" t="n">
+        <x:v>-100.3161126</x:v>
+      </x:c>
+      <x:c r="M448" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="N448" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O448" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P448" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="449">
+      <x:c r="A449" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B449" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C449" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D449" t="str">
+        <x:v>Crown - Acayucan</x:v>
+      </x:c>
+      <x:c r="E449" t="str">
+        <x:v>Beverage Packaging</x:v>
+      </x:c>
+      <x:c r="F449"/>
+      <x:c r="G449" t="str">
+        <x:v>Acayucan</x:v>
+      </x:c>
+      <x:c r="H449" t="str">
+        <x:v>VER</x:v>
+      </x:c>
+      <x:c r="I449"/>
+      <x:c r="J449" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="K449" t="n">
+        <x:v>17.949192</x:v>
+      </x:c>
+      <x:c r="L449" t="n">
+        <x:v>-94.9145974</x:v>
+      </x:c>
+      <x:c r="M449" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="N449" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O449" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P449" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="450">
+      <x:c r="A450" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B450" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C450" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D450" t="str">
+        <x:v>Crown - Amatlán de los Reyes</x:v>
+      </x:c>
+      <x:c r="E450" t="str">
+        <x:v>Transit Packaging</x:v>
+      </x:c>
+      <x:c r="F450"/>
+      <x:c r="G450" t="str">
+        <x:v>Amatlán de los Reyes</x:v>
+      </x:c>
+      <x:c r="H450" t="str">
+        <x:v>VER</x:v>
+      </x:c>
+      <x:c r="I450"/>
+      <x:c r="J450" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="K450" t="n">
+        <x:v>18.8426748</x:v>
+      </x:c>
+      <x:c r="L450" t="n">
+        <x:v>-96.9182301</x:v>
+      </x:c>
+      <x:c r="M450" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="N450" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O450" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P450" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="451">
+      <x:c r="A451" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B451" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C451" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="D451" t="str">
+        <x:v>Crown - Orizaba</x:v>
+      </x:c>
+      <x:c r="E451" t="str">
+        <x:v>Beverage Packaging</x:v>
+      </x:c>
+      <x:c r="F451"/>
+      <x:c r="G451" t="str">
+        <x:v>Orizaba</x:v>
+      </x:c>
+      <x:c r="H451" t="str">
+        <x:v>VER</x:v>
+      </x:c>
+      <x:c r="I451"/>
+      <x:c r="J451" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="K451" t="n">
+        <x:v>18.8504744</x:v>
+      </x:c>
+      <x:c r="L451" t="n">
+        <x:v>-97.1036396</x:v>
+      </x:c>
+      <x:c r="M451" t="str">
+        <x:v>Mexico</x:v>
+      </x:c>
+      <x:c r="N451" t="str">
+        <x:v>Verified - official Crown directory</x:v>
+      </x:c>
+      <x:c r="O451" t="str">
+        <x:v>https://www.crowncork.com/about/global-locations</x:v>
+      </x:c>
+      <x:c r="P451" t="str">
+        <x:v>Verified in Crown's current global-locations directory during the 2026-08-17 North America audit. Crown publishes a mapped city point rather than a street address.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -19973,7 +22143,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cfd8648d2684e89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Racb1fec058804ff6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20289,10 +22459,30 @@
         <x:v>Seven MCC locations retained separately. Arnold and Jacksonville are corroborated by current 2026 A-B announcements; the other five retain official network support but need fresh plant-specific confirmation.</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>Can Industry</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Crown Cork &amp; Seal</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>North America reconciled directly to Crown's current global-locations directory: 61 U.S. plants, 3 Canadian plants, and 9 Mexican plants. The Tampa corporate office is excluded.</x:v>
+      </x:c>
+      <x:c r="D16" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="E16" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>All 73 Crown North American production/packaging facilities are captured. Most newly added rows are Transit Packaging plants. Crown publishes city map points but not street addresses.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2287b0ba27b646c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2668c8537b584602"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20324,7 +22514,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
-        <x:v>Added verified or source-supported manufacturing, bottling, brewing, packaging, bakery, and agricultural production facilities across the United States, Canada, and Mexico, including national Coca-Cola, Grupo Bimbo, Aspire Bakeries, Mondelez, Molson Coors, and Anheuser-Busch audits; ordinary distribution-only sites remain excluded.</x:v>
+        <x:v>Added verified or source-supported manufacturing, bottling, brewing, packaging, bakery, and agricultural production facilities across the United States, Canada, and Mexico, including national Coca-Cola, Grupo Bimbo, Aspire Bakeries, Mondelez, Molson Coors, Anheuser-Busch, and Crown Cork &amp; Seal audits; ordinary distribution-only sites remain excluded.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15">
@@ -21668,16 +23858,16 @@
         <x:v>Crown - Benton</x:v>
       </x:c>
       <x:c r="C64" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D64" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E64" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F64" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Benton, AR, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -21688,16 +23878,16 @@
         <x:v>Crown - Dubuque</x:v>
       </x:c>
       <x:c r="C65" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D65" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E65" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F65" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Dubuque, IA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -21708,16 +23898,16 @@
         <x:v>Crown - Alsip</x:v>
       </x:c>
       <x:c r="C66" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D66" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E66" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F66" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Alsip, IL, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -21728,16 +23918,16 @@
         <x:v>Crown - Kankakee</x:v>
       </x:c>
       <x:c r="C67" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D67" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E67" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F67" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Kankakee, IL, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -21748,16 +23938,16 @@
         <x:v>Crown - Bowling Green</x:v>
       </x:c>
       <x:c r="C68" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D68" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E68" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F68" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Bowling Green, KY, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -21768,16 +23958,16 @@
         <x:v>Crown - Faribault</x:v>
       </x:c>
       <x:c r="C69" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D69" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E69" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F69" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Faribault, MN, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -21788,16 +23978,16 @@
         <x:v>Crown - Mankato</x:v>
       </x:c>
       <x:c r="C70" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D70" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E70" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F70" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Mankato, MN, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -21808,16 +23998,16 @@
         <x:v>Crown - Owatonna</x:v>
       </x:c>
       <x:c r="C71" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D71" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E71" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F71" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Owatonna, MN, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -21828,16 +24018,16 @@
         <x:v>Crown - Nichols</x:v>
       </x:c>
       <x:c r="C72" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D72" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E72" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F72" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Nichols, NY, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -21848,16 +24038,16 @@
         <x:v>Crown - Dayton</x:v>
       </x:c>
       <x:c r="C73" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D73" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E73" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F73" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Dayton, OH, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -21868,16 +24058,16 @@
         <x:v>Crown - Lancaster</x:v>
       </x:c>
       <x:c r="C74" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D74" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E74" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F74" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Lancaster, OH, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -21888,16 +24078,16 @@
         <x:v>Crown - Massillon</x:v>
       </x:c>
       <x:c r="C75" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D75" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E75" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F75" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Massillon, OH, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -21908,16 +24098,16 @@
         <x:v>Crown - Mill Park</x:v>
       </x:c>
       <x:c r="C76" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D76" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E76" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F76" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Mill Park, OH, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -21928,16 +24118,16 @@
         <x:v>Crown - Connellsville</x:v>
       </x:c>
       <x:c r="C77" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D77" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E77" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F77" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Connellsville, PA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -21948,16 +24138,16 @@
         <x:v>Crown - Hanover</x:v>
       </x:c>
       <x:c r="C78" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D78" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E78" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F78" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Hanover, PA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -21968,16 +24158,16 @@
         <x:v>Crown - Cheraw</x:v>
       </x:c>
       <x:c r="C79" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D79" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E79" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F79" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Cheraw, SC, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="28">
@@ -21991,13 +24181,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D80" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Crown directory map with longitude sign correction</x:v>
       </x:c>
       <x:c r="E80" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F80" s="23" t="str">
-        <x:v>Effingham, South Carolina; GeoNames ID 4577612</x:v>
+        <x:v>Effingham, SC, United States; Crown page displays a positive longitude in error; corrected to -79.7534</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -22008,16 +24198,16 @@
         <x:v>Crown - Conroe</x:v>
       </x:c>
       <x:c r="C81" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D81" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E81" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F81" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Conroe, TX, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -22028,16 +24218,16 @@
         <x:v>Crown - Ft. Bend</x:v>
       </x:c>
       <x:c r="C82" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D82" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E82" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F82" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Ft. Bend, TX, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -22048,16 +24238,16 @@
         <x:v>Crown - Martinsville</x:v>
       </x:c>
       <x:c r="C83" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D83" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E83" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F83" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Martinsville, VA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -22068,16 +24258,16 @@
         <x:v>Crown - Winchester</x:v>
       </x:c>
       <x:c r="C84" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D84" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E84" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F84" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Winchester, VA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -22088,16 +24278,16 @@
         <x:v>Crown - Olympia</x:v>
       </x:c>
       <x:c r="C85" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D85" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E85" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F85" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Olympia, WA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -22108,16 +24298,16 @@
         <x:v>Crown - La Crosse</x:v>
       </x:c>
       <x:c r="C86" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D86" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E86" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F86" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>La Crosse, WI, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -22128,16 +24318,16 @@
         <x:v>Crown - Worland</x:v>
       </x:c>
       <x:c r="C87" s="22" t="str">
-        <x:v>Retained</x:v>
+        <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D87" s="22" t="str">
-        <x:v>Official Crown global-locations page</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E87" s="22" t="str">
-        <x:v>Official city-level point</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F87" s="23" t="str">
-        <x:v>Matches Crown's published city coordinate; not verified as an exact building point</x:v>
+        <x:v>Worland, WY, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="28">
@@ -22151,13 +24341,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D88" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E88" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F88" s="23" t="str">
-        <x:v>Calgary, Alberta; GeoNames ID 5913490</x:v>
+        <x:v>Calgary, AB, Canada; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="28">
@@ -22171,13 +24361,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D89" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E89" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F89" s="23" t="str">
-        <x:v>Halton Hills, Ontario; GeoNames ID 5969721</x:v>
+        <x:v>Halton Hills, ON, Canada; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="28">
@@ -22191,13 +24381,13 @@
         <x:v>Added — approximate</x:v>
       </x:c>
       <x:c r="D90" s="22" t="str">
-        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+        <x:v>Crown official global-locations map</x:v>
       </x:c>
       <x:c r="E90" s="22" t="str">
-        <x:v>City-center fallback</x:v>
+        <x:v>Official directory city point</x:v>
       </x:c>
       <x:c r="F90" s="23" t="str">
-        <x:v>Toronto, Ontario; GeoNames ID 6167865</x:v>
+        <x:v>Toronto, ON, Canada; exact plant coordinate should replace this official directory point when independently verified</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -28500,10 +30690,930 @@
         <x:v>3723 County Road 905, Jonesboro, AR 72401; Arkansas DEQ NAD83 GPS</x:v>
       </x:c>
     </x:row>
+    <x:row r="406">
+      <x:c r="A406" t="n">
+        <x:v>406</x:v>
+      </x:c>
+      <x:c r="B406" t="str">
+        <x:v>Crown - Fordyce</x:v>
+      </x:c>
+      <x:c r="C406" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D406" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E406" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F406" t="str">
+        <x:v>Fordyce, AR, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="407">
+      <x:c r="A407" t="n">
+        <x:v>407</x:v>
+      </x:c>
+      <x:c r="B407" t="str">
+        <x:v>Crown - Sheridan</x:v>
+      </x:c>
+      <x:c r="C407" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D407" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E407" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F407" t="str">
+        <x:v>Sheridan, AR, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="408">
+      <x:c r="A408" t="n">
+        <x:v>408</x:v>
+      </x:c>
+      <x:c r="B408" t="str">
+        <x:v>Crown - Phoenix</x:v>
+      </x:c>
+      <x:c r="C408" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D408" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E408" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F408" t="str">
+        <x:v>Phoenix, AZ, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="409">
+      <x:c r="A409" t="n">
+        <x:v>409</x:v>
+      </x:c>
+      <x:c r="B409" t="str">
+        <x:v>Crown - Bay Point</x:v>
+      </x:c>
+      <x:c r="C409" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D409" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E409" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F409" t="str">
+        <x:v>Bay Point, CA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="410">
+      <x:c r="A410" t="n">
+        <x:v>410</x:v>
+      </x:c>
+      <x:c r="B410" t="str">
+        <x:v>Crown - Stockton</x:v>
+      </x:c>
+      <x:c r="C410" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D410" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E410" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F410" t="str">
+        <x:v>Stockton, CA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="411">
+      <x:c r="A411" t="n">
+        <x:v>411</x:v>
+      </x:c>
+      <x:c r="B411" t="str">
+        <x:v>Crown - Douglasville</x:v>
+      </x:c>
+      <x:c r="C411" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D411" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E411" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F411" t="str">
+        <x:v>Douglasville, GA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="412">
+      <x:c r="A412" t="n">
+        <x:v>412</x:v>
+      </x:c>
+      <x:c r="B412" t="str">
+        <x:v>Crown - LaGrange</x:v>
+      </x:c>
+      <x:c r="C412" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D412" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E412" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F412" t="str">
+        <x:v>LaGrange, GA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="413">
+      <x:c r="A413" t="n">
+        <x:v>413</x:v>
+      </x:c>
+      <x:c r="B413" t="str">
+        <x:v>Crown - Macon</x:v>
+      </x:c>
+      <x:c r="C413" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D413" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E413" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F413" t="str">
+        <x:v>Macon, GA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="414">
+      <x:c r="A414" t="n">
+        <x:v>414</x:v>
+      </x:c>
+      <x:c r="B414" t="str">
+        <x:v>Crown - Bridgeview</x:v>
+      </x:c>
+      <x:c r="C414" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D414" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E414" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F414" t="str">
+        <x:v>Bridgeview, IL, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="415">
+      <x:c r="A415" t="n">
+        <x:v>415</x:v>
+      </x:c>
+      <x:c r="B415" t="str">
+        <x:v>Crown - Dixmoor</x:v>
+      </x:c>
+      <x:c r="C415" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D415" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E415" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F415" t="str">
+        <x:v>Dixmoor, IL, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="416">
+      <x:c r="A416" t="n">
+        <x:v>416</x:v>
+      </x:c>
+      <x:c r="B416" t="str">
+        <x:v>Crown - Roselle</x:v>
+      </x:c>
+      <x:c r="C416" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D416" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E416" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F416" t="str">
+        <x:v>Roselle, IL, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="417">
+      <x:c r="A417" t="n">
+        <x:v>417</x:v>
+      </x:c>
+      <x:c r="B417" t="str">
+        <x:v>Crown - Elkhart</x:v>
+      </x:c>
+      <x:c r="C417" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D417" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E417" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F417" t="str">
+        <x:v>Elkhart, IN, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="418">
+      <x:c r="A418" t="n">
+        <x:v>418</x:v>
+      </x:c>
+      <x:c r="B418" t="str">
+        <x:v>Crown - Gary</x:v>
+      </x:c>
+      <x:c r="C418" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D418" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E418" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F418" t="str">
+        <x:v>Gary, IN, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="419">
+      <x:c r="A419" t="n">
+        <x:v>419</x:v>
+      </x:c>
+      <x:c r="B419" t="str">
+        <x:v>Crown - Florence</x:v>
+      </x:c>
+      <x:c r="C419" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D419" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E419" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F419" t="str">
+        <x:v>Florence, KY, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="420">
+      <x:c r="A420" t="n">
+        <x:v>420</x:v>
+      </x:c>
+      <x:c r="B420" t="str">
+        <x:v>Crown - Monroe</x:v>
+      </x:c>
+      <x:c r="C420" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D420" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E420" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F420" t="str">
+        <x:v>Monroe, LA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="421">
+      <x:c r="A421" t="n">
+        <x:v>421</x:v>
+      </x:c>
+      <x:c r="B421" t="str">
+        <x:v>Crown - Belcamp</x:v>
+      </x:c>
+      <x:c r="C421" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D421" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E421" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F421" t="str">
+        <x:v>Belcamp, MD, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="422">
+      <x:c r="A422" t="n">
+        <x:v>422</x:v>
+      </x:c>
+      <x:c r="B422" t="str">
+        <x:v>Crown - Brighton</x:v>
+      </x:c>
+      <x:c r="C422" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D422" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E422" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F422" t="str">
+        <x:v>Brighton, MI, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="423">
+      <x:c r="A423" t="n">
+        <x:v>423</x:v>
+      </x:c>
+      <x:c r="B423" t="str">
+        <x:v>Crown - Eden</x:v>
+      </x:c>
+      <x:c r="C423" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D423" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E423" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F423" t="str">
+        <x:v>Eden, NC, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="424">
+      <x:c r="A424" t="n">
+        <x:v>424</x:v>
+      </x:c>
+      <x:c r="B424" t="str">
+        <x:v>Crown - Salisbury</x:v>
+      </x:c>
+      <x:c r="C424" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D424" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E424" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F424" t="str">
+        <x:v>Salisbury, NC, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="425">
+      <x:c r="A425" t="n">
+        <x:v>425</x:v>
+      </x:c>
+      <x:c r="B425" t="str">
+        <x:v>Crown - Irvington</x:v>
+      </x:c>
+      <x:c r="C425" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D425" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E425" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F425" t="str">
+        <x:v>Irvington, NJ, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="426">
+      <x:c r="A426" t="n">
+        <x:v>426</x:v>
+      </x:c>
+      <x:c r="B426" t="str">
+        <x:v>Crown - Mesquite</x:v>
+      </x:c>
+      <x:c r="C426" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D426" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E426" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F426" t="str">
+        <x:v>Mesquite, NV, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="427">
+      <x:c r="A427" t="n">
+        <x:v>427</x:v>
+      </x:c>
+      <x:c r="B427" t="str">
+        <x:v>Crown - Cleveland</x:v>
+      </x:c>
+      <x:c r="C427" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D427" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E427" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F427" t="str">
+        <x:v>Cleveland, OH, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="428">
+      <x:c r="A428" t="n">
+        <x:v>428</x:v>
+      </x:c>
+      <x:c r="B428" t="str">
+        <x:v>Crown - Loveland</x:v>
+      </x:c>
+      <x:c r="C428" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D428" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E428" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F428" t="str">
+        <x:v>Loveland, OH, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="429">
+      <x:c r="A429" t="n">
+        <x:v>429</x:v>
+      </x:c>
+      <x:c r="B429" t="str">
+        <x:v>Crown - West Chester</x:v>
+      </x:c>
+      <x:c r="C429" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D429" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E429" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F429" t="str">
+        <x:v>West Chester, OH, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="430">
+      <x:c r="A430" t="n">
+        <x:v>430</x:v>
+      </x:c>
+      <x:c r="B430" t="str">
+        <x:v>Crown - Hazleton</x:v>
+      </x:c>
+      <x:c r="C430" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D430" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E430" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F430" t="str">
+        <x:v>Hazleton, PA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="431">
+      <x:c r="A431" t="n">
+        <x:v>431</x:v>
+      </x:c>
+      <x:c r="B431" t="str">
+        <x:v>Crown - South Canaan</x:v>
+      </x:c>
+      <x:c r="C431" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D431" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E431" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F431" t="str">
+        <x:v>South Canaan, PA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="432">
+      <x:c r="A432" t="n">
+        <x:v>432</x:v>
+      </x:c>
+      <x:c r="B432" t="str">
+        <x:v>Crown - East Providence</x:v>
+      </x:c>
+      <x:c r="C432" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D432" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E432" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F432" t="str">
+        <x:v>East Providence, RI, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="433">
+      <x:c r="A433" t="n">
+        <x:v>433</x:v>
+      </x:c>
+      <x:c r="B433" t="str">
+        <x:v>Crown - Darlington</x:v>
+      </x:c>
+      <x:c r="C433" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D433" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E433" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F433" t="str">
+        <x:v>Darlington, SC, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="434">
+      <x:c r="A434" t="n">
+        <x:v>434</x:v>
+      </x:c>
+      <x:c r="B434" t="str">
+        <x:v>Crown - Greer</x:v>
+      </x:c>
+      <x:c r="C434" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D434" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E434" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F434" t="str">
+        <x:v>Greer, SC, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="435">
+      <x:c r="A435" t="n">
+        <x:v>435</x:v>
+      </x:c>
+      <x:c r="B435" t="str">
+        <x:v>Crown - Latta</x:v>
+      </x:c>
+      <x:c r="C435" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D435" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E435" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F435" t="str">
+        <x:v>Latta, SC, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="436">
+      <x:c r="A436" t="n">
+        <x:v>436</x:v>
+      </x:c>
+      <x:c r="B436" t="str">
+        <x:v>Crown - Spartanburg</x:v>
+      </x:c>
+      <x:c r="C436" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D436" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E436" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F436" t="str">
+        <x:v>Spartanburg, SC, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="437">
+      <x:c r="A437" t="n">
+        <x:v>437</x:v>
+      </x:c>
+      <x:c r="B437" t="str">
+        <x:v>Crown - Orange</x:v>
+      </x:c>
+      <x:c r="C437" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D437" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E437" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F437" t="str">
+        <x:v>Orange, TX, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="438">
+      <x:c r="A438" t="n">
+        <x:v>438</x:v>
+      </x:c>
+      <x:c r="B438" t="str">
+        <x:v>Crown - San Antonio</x:v>
+      </x:c>
+      <x:c r="C438" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D438" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E438" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F438" t="str">
+        <x:v>San Antonio, TX, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="439">
+      <x:c r="A439" t="n">
+        <x:v>439</x:v>
+      </x:c>
+      <x:c r="B439" t="str">
+        <x:v>Crown - Forest</x:v>
+      </x:c>
+      <x:c r="C439" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D439" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E439" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F439" t="str">
+        <x:v>Forest, VA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="440">
+      <x:c r="A440" t="n">
+        <x:v>440</x:v>
+      </x:c>
+      <x:c r="B440" t="str">
+        <x:v>Crown - Danville</x:v>
+      </x:c>
+      <x:c r="C440" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D440" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E440" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F440" t="str">
+        <x:v>Danville, WA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="441">
+      <x:c r="A441" t="n">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="B441" t="str">
+        <x:v>Crown - Woodland</x:v>
+      </x:c>
+      <x:c r="C441" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D441" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E441" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F441" t="str">
+        <x:v>Woodland, WA, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="442">
+      <x:c r="A442" t="n">
+        <x:v>442</x:v>
+      </x:c>
+      <x:c r="B442" t="str">
+        <x:v>Crown - Oshkosh</x:v>
+      </x:c>
+      <x:c r="C442" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D442" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E442" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F442" t="str">
+        <x:v>Oshkosh, WI, United States; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="443">
+      <x:c r="A443" t="n">
+        <x:v>443</x:v>
+      </x:c>
+      <x:c r="B443" t="str">
+        <x:v>Crown - Ensenada</x:v>
+      </x:c>
+      <x:c r="C443" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D443" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E443" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F443" t="str">
+        <x:v>Ensenada, BCN, Mexico; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="444">
+      <x:c r="A444" t="n">
+        <x:v>444</x:v>
+      </x:c>
+      <x:c r="B444" t="str">
+        <x:v>Crown - Chihuahua</x:v>
+      </x:c>
+      <x:c r="C444" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D444" t="str">
+        <x:v>GeoNames city/place centroid (CC BY 4.0)</x:v>
+      </x:c>
+      <x:c r="E444" t="str">
+        <x:v>City-center fallback</x:v>
+      </x:c>
+      <x:c r="F444" t="str">
+        <x:v>Chihuahua, CHH, Mexico; GeoNames coordinate 28.6352778, -106.0888889; Crown directory longitude is erroneous</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="445">
+      <x:c r="A445" t="n">
+        <x:v>445</x:v>
+      </x:c>
+      <x:c r="B445" t="str">
+        <x:v>Crown - Guadalajara</x:v>
+      </x:c>
+      <x:c r="C445" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D445" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E445" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F445" t="str">
+        <x:v>Guadalajara, JAL, Mexico; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="446">
+      <x:c r="A446" t="n">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="B446" t="str">
+        <x:v>Crown - Toluca</x:v>
+      </x:c>
+      <x:c r="C446" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D446" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E446" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F446" t="str">
+        <x:v>Toluca, MEX, Mexico; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="447">
+      <x:c r="A447" t="n">
+        <x:v>447</x:v>
+      </x:c>
+      <x:c r="B447" t="str">
+        <x:v>Crown - Ciénega de Flores</x:v>
+      </x:c>
+      <x:c r="C447" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D447" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E447" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F447" t="str">
+        <x:v>Ciénega de Flores, NLE, Mexico; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="448">
+      <x:c r="A448" t="n">
+        <x:v>448</x:v>
+      </x:c>
+      <x:c r="B448" t="str">
+        <x:v>Crown - Monterrey</x:v>
+      </x:c>
+      <x:c r="C448" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D448" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E448" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F448" t="str">
+        <x:v>Monterrey, NLE, Mexico; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="449">
+      <x:c r="A449" t="n">
+        <x:v>449</x:v>
+      </x:c>
+      <x:c r="B449" t="str">
+        <x:v>Crown - Acayucan</x:v>
+      </x:c>
+      <x:c r="C449" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D449" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E449" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F449" t="str">
+        <x:v>Acayucan, VER, Mexico; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="450">
+      <x:c r="A450" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="B450" t="str">
+        <x:v>Crown - Amatlán de los Reyes</x:v>
+      </x:c>
+      <x:c r="C450" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D450" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E450" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F450" t="str">
+        <x:v>Amatlán de los Reyes, VER, Mexico; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="451">
+      <x:c r="A451" t="n">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="B451" t="str">
+        <x:v>Crown - Orizaba</x:v>
+      </x:c>
+      <x:c r="C451" t="str">
+        <x:v>Added — approximate</x:v>
+      </x:c>
+      <x:c r="D451" t="str">
+        <x:v>Crown official global-locations map</x:v>
+      </x:c>
+      <x:c r="E451" t="str">
+        <x:v>Official directory city point</x:v>
+      </x:c>
+      <x:c r="F451" t="str">
+        <x:v>Orizaba, VER, Mexico; exact plant coordinate should replace this official directory point when independently verified</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0901bf7b2be640c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra406aec30af54b77"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>